<commit_message>
Rebuild the site as real pages: menu, categories, builder, order, about, FAQ
The one-page ordering panel is replaced by separate pages, so the browser's
Back returns a customer to exactly where they were.

- menu.html: one door per category; menu/<category>.html: dish cards with
  size, quantity and Add on the card, sticky category rail
- build.html: build your own, customize a specialty pizza (extra toppings
  priced per size), or fill a deal's pizzas one after another
- order.html: lines, quantities, special instructions, totals, checkout
- about.html, faq.html (answers built from the shop's data, plus a new
  Questions sheet in the workbook), shared header and footer
- shared tasty.css / tasty.js with content-hashed URLs; audit checks every page

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TastyPizza-Control.xlsx
+++ b/TastyPizza-Control.xlsx
@@ -14,7 +14,8 @@
     <sheet name="Pizza builder" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Hours" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Shop details" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Lists" sheetId="8" state="hidden" r:id="rId8"/>
+    <sheet name="Questions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Lists" sheetId="9" state="hidden" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6628,6 +6629,93 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Questions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Extra questions for the FAQ page. Hours, delivery areas, crusts and vegetarian pizzas are answered automatically from the other sheets. Fill a blank row to add one; clear a row to remove it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Answer</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="n"/>
+      <c r="B5" s="10" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="n"/>
+      <c r="B6" s="10" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="n"/>
+      <c r="B7" s="10" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="n"/>
+      <c r="B8" s="10" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="10" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="n"/>
+      <c r="B10" s="10" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="10" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="10" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Client round 3: drinks, add-ons, special toppings, half toppings, hours, crusts, delivery
- Drinks page with the six beverages
- Cheese / extra meat tick boxes on donair and sub cards, priced by size
- Builder: extra cheese and the special toppings, each priced by size;
  left half / whole / right half under any chosen topping (whole by default)
  with a note about the extra labour charge
- Saturday closes at midnight; gluten-free crust $6.45; whole wheat removed
- Delivery areas updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TastyPizza-Control.xlsx
+++ b/TastyPizza-Control.xlsx
@@ -1228,7 +1228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J155"/>
+  <dimension ref="A1:J161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="E24" s="10" t="n">
-        <v>4.99</v>
+        <v>6.45</v>
       </c>
       <c r="F24" s="10" t="n"/>
       <c r="G24" s="10" t="n"/>
@@ -4118,52 +4118,48 @@
     <row r="89">
       <c r="A89" s="9" t="inlineStr">
         <is>
-          <t>fish/Fish &amp; Chips — 1 pc</t>
+          <t>beverages/Any 519ml Pop</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t>Fish &amp; Chips</t>
+          <t>Cold Drinks</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
         <is>
-          <t>Fish &amp; Chips — 1 pc</t>
+          <t>Any 519ml Pop</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr"/>
       <c r="E89" s="10" t="n">
-        <v>11.95</v>
+        <v>2.59</v>
       </c>
       <c r="F89" s="10" t="n"/>
       <c r="G89" s="10" t="n"/>
       <c r="H89" s="10" t="n"/>
       <c r="I89" s="10" t="inlineStr"/>
-      <c r="J89" s="10" t="inlineStr">
-        <is>
-          <t>fish-and-chips</t>
-        </is>
-      </c>
+      <c r="J89" s="10" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="9" t="inlineStr">
         <is>
-          <t>fish/Fish &amp; Chips — 2 pc</t>
+          <t>beverages/Any Juice, Gatorade, G2 or Energy Drink</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t>Fish &amp; Chips</t>
+          <t>Cold Drinks</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
         <is>
-          <t>Fish &amp; Chips — 2 pc</t>
+          <t>Any Juice, Gatorade, G2 or Energy Drink</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr"/>
       <c r="E90" s="10" t="n">
-        <v>15.95</v>
+        <v>3.39</v>
       </c>
       <c r="F90" s="10" t="n"/>
       <c r="G90" s="10" t="n"/>
@@ -4174,22 +4170,22 @@
     <row r="91">
       <c r="A91" s="9" t="inlineStr">
         <is>
-          <t>fish/Fish &amp; Chips — 3 pc</t>
+          <t>beverages/Chocolate Milk</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
         <is>
-          <t>Fish &amp; Chips</t>
+          <t>Cold Drinks</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
         <is>
-          <t>Fish &amp; Chips — 3 pc</t>
+          <t>Chocolate Milk</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr"/>
       <c r="E91" s="10" t="n">
-        <v>17.95</v>
+        <v>2.79</v>
       </c>
       <c r="F91" s="10" t="n"/>
       <c r="G91" s="10" t="n"/>
@@ -4200,22 +4196,22 @@
     <row r="92">
       <c r="A92" s="9" t="inlineStr">
         <is>
-          <t>fish/Extra Piece of Fish</t>
+          <t>beverages/Any 355ml Pop</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t>Fish &amp; Chips</t>
+          <t>Cold Drinks</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
         <is>
-          <t>Extra Piece of Fish</t>
+          <t>Any 355ml Pop</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr"/>
       <c r="E92" s="10" t="n">
-        <v>4.95</v>
+        <v>1.59</v>
       </c>
       <c r="F92" s="10" t="n"/>
       <c r="G92" s="10" t="n"/>
@@ -4226,26 +4222,22 @@
     <row r="93">
       <c r="A93" s="9" t="inlineStr">
         <is>
-          <t>fish/Fish Family Pack</t>
+          <t>beverages/Any 2L Pop</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
         <is>
-          <t>Fish &amp; Chips</t>
+          <t>Cold Drinks</t>
         </is>
       </c>
       <c r="C93" s="10" t="inlineStr">
         <is>
-          <t>Fish Family Pack</t>
-        </is>
-      </c>
-      <c r="D93" s="10" t="inlineStr">
-        <is>
-          <t>10 pieces of fish, 2 large fries, large gravy, coleslaw and tartar sauce.</t>
-        </is>
-      </c>
+          <t>Any 2L Pop</t>
+        </is>
+      </c>
+      <c r="D93" s="10" t="inlineStr"/>
       <c r="E93" s="10" t="n">
-        <v>46.95</v>
+        <v>4.19</v>
       </c>
       <c r="F93" s="10" t="n"/>
       <c r="G93" s="10" t="n"/>
@@ -4256,124 +4248,104 @@
     <row r="94">
       <c r="A94" s="9" t="inlineStr">
         <is>
-          <t>seafood/Scallops &amp; Chips</t>
+          <t>beverages/Aquafina Water 591ml</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t>More Seafood</t>
+          <t>Cold Drinks</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
         <is>
-          <t>Scallops &amp; Chips</t>
-        </is>
-      </c>
-      <c r="D94" s="10" t="inlineStr">
-        <is>
-          <t>10 scallops.</t>
-        </is>
-      </c>
+          <t>Aquafina Water 591ml</t>
+        </is>
+      </c>
+      <c r="D94" s="10" t="inlineStr"/>
       <c r="E94" s="10" t="n">
-        <v>14.95</v>
+        <v>1.69</v>
       </c>
       <c r="F94" s="10" t="n"/>
       <c r="G94" s="10" t="n"/>
       <c r="H94" s="10" t="n"/>
       <c r="I94" s="10" t="inlineStr"/>
-      <c r="J94" s="10" t="inlineStr">
-        <is>
-          <t>scallops</t>
-        </is>
-      </c>
+      <c r="J94" s="10" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="9" t="inlineStr">
         <is>
-          <t>seafood/Clams &amp; Chips</t>
+          <t>fish/Fish &amp; Chips — 1 pc</t>
         </is>
       </c>
       <c r="B95" s="10" t="inlineStr">
         <is>
-          <t>More Seafood</t>
+          <t>Fish &amp; Chips</t>
         </is>
       </c>
       <c r="C95" s="10" t="inlineStr">
         <is>
-          <t>Clams &amp; Chips</t>
-        </is>
-      </c>
-      <c r="D95" s="10" t="inlineStr">
-        <is>
-          <t>Two cups of clams.</t>
-        </is>
-      </c>
+          <t>Fish &amp; Chips — 1 pc</t>
+        </is>
+      </c>
+      <c r="D95" s="10" t="inlineStr"/>
       <c r="E95" s="10" t="n">
-        <v>14.95</v>
+        <v>11.95</v>
       </c>
       <c r="F95" s="10" t="n"/>
       <c r="G95" s="10" t="n"/>
       <c r="H95" s="10" t="n"/>
       <c r="I95" s="10" t="inlineStr"/>
-      <c r="J95" s="10" t="inlineStr"/>
+      <c r="J95" s="10" t="inlineStr">
+        <is>
+          <t>fish-and-chips</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="9" t="inlineStr">
         <is>
-          <t>seafood/Shrimp &amp; Chips</t>
+          <t>fish/Fish &amp; Chips — 2 pc</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
         <is>
-          <t>More Seafood</t>
+          <t>Fish &amp; Chips</t>
         </is>
       </c>
       <c r="C96" s="10" t="inlineStr">
         <is>
-          <t>Shrimp &amp; Chips</t>
-        </is>
-      </c>
-      <c r="D96" s="10" t="inlineStr">
-        <is>
-          <t>12 shrimp.</t>
-        </is>
-      </c>
+          <t>Fish &amp; Chips — 2 pc</t>
+        </is>
+      </c>
+      <c r="D96" s="10" t="inlineStr"/>
       <c r="E96" s="10" t="n">
-        <v>14.95</v>
+        <v>15.95</v>
       </c>
       <c r="F96" s="10" t="n"/>
       <c r="G96" s="10" t="n"/>
       <c r="H96" s="10" t="n"/>
       <c r="I96" s="10" t="inlineStr"/>
-      <c r="J96" s="10" t="inlineStr">
-        <is>
-          <t>shrimp</t>
-        </is>
-      </c>
+      <c r="J96" s="10" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="9" t="inlineStr">
         <is>
-          <t>seafood/Seafood Platter</t>
+          <t>fish/Fish &amp; Chips — 3 pc</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
         <is>
-          <t>More Seafood</t>
+          <t>Fish &amp; Chips</t>
         </is>
       </c>
       <c r="C97" s="10" t="inlineStr">
         <is>
-          <t>Seafood Platter</t>
-        </is>
-      </c>
-      <c r="D97" s="10" t="inlineStr">
-        <is>
-          <t>A piece of fish, fries, 5 scallops, 5 shrimp and clams.</t>
-        </is>
-      </c>
+          <t>Fish &amp; Chips — 3 pc</t>
+        </is>
+      </c>
+      <c r="D97" s="10" t="inlineStr"/>
       <c r="E97" s="10" t="n">
-        <v>23.95</v>
+        <v>17.95</v>
       </c>
       <c r="F97" s="10" t="n"/>
       <c r="G97" s="10" t="n"/>
@@ -4384,22 +4356,22 @@
     <row r="98">
       <c r="A98" s="9" t="inlineStr">
         <is>
-          <t>seafood/Extra Coleslaw — Small</t>
+          <t>fish/Extra Piece of Fish</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t>More Seafood</t>
+          <t>Fish &amp; Chips</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
         <is>
-          <t>Extra Coleslaw — Small</t>
+          <t>Extra Piece of Fish</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr"/>
       <c r="E98" s="10" t="n">
-        <v>2.25</v>
+        <v>4.95</v>
       </c>
       <c r="F98" s="10" t="n"/>
       <c r="G98" s="10" t="n"/>
@@ -4410,22 +4382,26 @@
     <row r="99">
       <c r="A99" s="9" t="inlineStr">
         <is>
-          <t>seafood/Extra Coleslaw — Large</t>
+          <t>fish/Fish Family Pack</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t>More Seafood</t>
+          <t>Fish &amp; Chips</t>
         </is>
       </c>
       <c r="C99" s="10" t="inlineStr">
         <is>
-          <t>Extra Coleslaw — Large</t>
-        </is>
-      </c>
-      <c r="D99" s="10" t="inlineStr"/>
+          <t>Fish Family Pack</t>
+        </is>
+      </c>
+      <c r="D99" s="10" t="inlineStr">
+        <is>
+          <t>10 pieces of fish, 2 large fries, large gravy, coleslaw and tartar sauce.</t>
+        </is>
+      </c>
       <c r="E99" s="10" t="n">
-        <v>3.45</v>
+        <v>46.95</v>
       </c>
       <c r="F99" s="10" t="n"/>
       <c r="G99" s="10" t="n"/>
@@ -4436,207 +4412,187 @@
     <row r="100">
       <c r="A100" s="9" t="inlineStr">
         <is>
-          <t>subs/Cold Cut</t>
+          <t>seafood/Scallops &amp; Chips</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t>Subs</t>
+          <t>More Seafood</t>
         </is>
       </c>
       <c r="C100" s="10" t="inlineStr">
         <is>
-          <t>Cold Cut</t>
-        </is>
-      </c>
-      <c r="D100" s="10" t="inlineStr"/>
+          <t>Scallops &amp; Chips</t>
+        </is>
+      </c>
+      <c r="D100" s="10" t="inlineStr">
+        <is>
+          <t>10 scallops.</t>
+        </is>
+      </c>
       <c r="E100" s="10" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="F100" s="10" t="n">
-        <v>13.25</v>
-      </c>
+        <v>14.95</v>
+      </c>
+      <c r="F100" s="10" t="n"/>
       <c r="G100" s="10" t="n"/>
       <c r="H100" s="10" t="n"/>
-      <c r="I100" s="10" t="inlineStr">
-        <is>
-          <t>Small / Large</t>
-        </is>
-      </c>
+      <c r="I100" s="10" t="inlineStr"/>
       <c r="J100" s="10" t="inlineStr">
         <is>
-          <t>cold-cut-sub</t>
+          <t>scallops</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="9" t="inlineStr">
         <is>
-          <t>subs/Salami &amp; Ham</t>
+          <t>seafood/Clams &amp; Chips</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t>Subs</t>
+          <t>More Seafood</t>
         </is>
       </c>
       <c r="C101" s="10" t="inlineStr">
         <is>
-          <t>Salami &amp; Ham</t>
-        </is>
-      </c>
-      <c r="D101" s="10" t="inlineStr"/>
+          <t>Clams &amp; Chips</t>
+        </is>
+      </c>
+      <c r="D101" s="10" t="inlineStr">
+        <is>
+          <t>Two cups of clams.</t>
+        </is>
+      </c>
       <c r="E101" s="10" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="F101" s="10" t="n">
-        <v>13.25</v>
-      </c>
+        <v>14.95</v>
+      </c>
+      <c r="F101" s="10" t="n"/>
       <c r="G101" s="10" t="n"/>
       <c r="H101" s="10" t="n"/>
-      <c r="I101" s="10" t="inlineStr">
-        <is>
-          <t>Small / Large</t>
-        </is>
-      </c>
+      <c r="I101" s="10" t="inlineStr"/>
       <c r="J101" s="10" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="9" t="inlineStr">
         <is>
-          <t>subs/Pizza Sub</t>
+          <t>seafood/Shrimp &amp; Chips</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t>Subs</t>
+          <t>More Seafood</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
         <is>
-          <t>Pizza Sub</t>
-        </is>
-      </c>
-      <c r="D102" s="10" t="inlineStr"/>
+          <t>Shrimp &amp; Chips</t>
+        </is>
+      </c>
+      <c r="D102" s="10" t="inlineStr">
+        <is>
+          <t>12 shrimp.</t>
+        </is>
+      </c>
       <c r="E102" s="10" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="F102" s="10" t="n">
-        <v>13.25</v>
-      </c>
+        <v>14.95</v>
+      </c>
+      <c r="F102" s="10" t="n"/>
       <c r="G102" s="10" t="n"/>
       <c r="H102" s="10" t="n"/>
-      <c r="I102" s="10" t="inlineStr">
-        <is>
-          <t>Small / Large</t>
-        </is>
-      </c>
-      <c r="J102" s="10" t="inlineStr"/>
+      <c r="I102" s="10" t="inlineStr"/>
+      <c r="J102" s="10" t="inlineStr">
+        <is>
+          <t>shrimp</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="9" t="inlineStr">
         <is>
-          <t>subs/Vegetarian</t>
+          <t>seafood/Seafood Platter</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t>Subs</t>
+          <t>More Seafood</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
         <is>
-          <t>Vegetarian</t>
-        </is>
-      </c>
-      <c r="D103" s="10" t="inlineStr"/>
+          <t>Seafood Platter</t>
+        </is>
+      </c>
+      <c r="D103" s="10" t="inlineStr">
+        <is>
+          <t>A piece of fish, fries, 5 scallops, 5 shrimp and clams.</t>
+        </is>
+      </c>
       <c r="E103" s="10" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="F103" s="10" t="n">
-        <v>13.25</v>
-      </c>
+        <v>23.95</v>
+      </c>
+      <c r="F103" s="10" t="n"/>
       <c r="G103" s="10" t="n"/>
       <c r="H103" s="10" t="n"/>
-      <c r="I103" s="10" t="inlineStr">
-        <is>
-          <t>Small / Large</t>
-        </is>
-      </c>
+      <c r="I103" s="10" t="inlineStr"/>
       <c r="J103" s="10" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="9" t="inlineStr">
         <is>
-          <t>subs/Real Turkey</t>
+          <t>seafood/Extra Coleslaw — Small</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t>Subs</t>
+          <t>More Seafood</t>
         </is>
       </c>
       <c r="C104" s="10" t="inlineStr">
         <is>
-          <t>Real Turkey</t>
+          <t>Extra Coleslaw — Small</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr"/>
       <c r="E104" s="10" t="n">
-        <v>11.45</v>
-      </c>
-      <c r="F104" s="10" t="n">
-        <v>13.25</v>
-      </c>
+        <v>2.25</v>
+      </c>
+      <c r="F104" s="10" t="n"/>
       <c r="G104" s="10" t="n"/>
       <c r="H104" s="10" t="n"/>
-      <c r="I104" s="10" t="inlineStr">
-        <is>
-          <t>Small / Large</t>
-        </is>
-      </c>
+      <c r="I104" s="10" t="inlineStr"/>
       <c r="J104" s="10" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="9" t="inlineStr">
         <is>
-          <t>subs/Bubba</t>
+          <t>seafood/Extra Coleslaw — Large</t>
         </is>
       </c>
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t>Subs</t>
+          <t>More Seafood</t>
         </is>
       </c>
       <c r="C105" s="10" t="inlineStr">
         <is>
-          <t>Bubba</t>
-        </is>
-      </c>
-      <c r="D105" s="10" t="inlineStr">
-        <is>
-          <t>The one people ask for by name.</t>
-        </is>
-      </c>
+          <t>Extra Coleslaw — Large</t>
+        </is>
+      </c>
+      <c r="D105" s="10" t="inlineStr"/>
       <c r="E105" s="10" t="n">
-        <v>11.95</v>
-      </c>
-      <c r="F105" s="10" t="n">
-        <v>14.25</v>
-      </c>
+        <v>3.45</v>
+      </c>
+      <c r="F105" s="10" t="n"/>
       <c r="G105" s="10" t="n"/>
       <c r="H105" s="10" t="n"/>
-      <c r="I105" s="10" t="inlineStr">
-        <is>
-          <t>Small / Large</t>
-        </is>
-      </c>
+      <c r="I105" s="10" t="inlineStr"/>
       <c r="J105" s="10" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="9" t="inlineStr">
         <is>
-          <t>subs/Club</t>
+          <t>subs/Cold Cut</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
@@ -4646,15 +4602,15 @@
       </c>
       <c r="C106" s="10" t="inlineStr">
         <is>
-          <t>Club</t>
+          <t>Cold Cut</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr"/>
       <c r="E106" s="10" t="n">
-        <v>11.95</v>
+        <v>10.95</v>
       </c>
       <c r="F106" s="10" t="n">
-        <v>14.25</v>
+        <v>13.25</v>
       </c>
       <c r="G106" s="10" t="n"/>
       <c r="H106" s="10" t="n"/>
@@ -4663,12 +4619,16 @@
           <t>Small / Large</t>
         </is>
       </c>
-      <c r="J106" s="10" t="inlineStr"/>
+      <c r="J106" s="10" t="inlineStr">
+        <is>
+          <t>cold-cut-sub</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="9" t="inlineStr">
         <is>
-          <t>subs/Steak</t>
+          <t>subs/Salami &amp; Ham</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
@@ -4678,15 +4638,15 @@
       </c>
       <c r="C107" s="10" t="inlineStr">
         <is>
-          <t>Steak</t>
+          <t>Salami &amp; Ham</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr"/>
       <c r="E107" s="10" t="n">
-        <v>11.95</v>
+        <v>10.95</v>
       </c>
       <c r="F107" s="10" t="n">
-        <v>14.95</v>
+        <v>13.25</v>
       </c>
       <c r="G107" s="10" t="n"/>
       <c r="H107" s="10" t="n"/>
@@ -4695,16 +4655,12 @@
           <t>Small / Large</t>
         </is>
       </c>
-      <c r="J107" s="10" t="inlineStr">
-        <is>
-          <t>steak-sub</t>
-        </is>
-      </c>
+      <c r="J107" s="10" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="9" t="inlineStr">
         <is>
-          <t>subs/Donair Sub</t>
+          <t>subs/Pizza Sub</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
@@ -4714,15 +4670,15 @@
       </c>
       <c r="C108" s="10" t="inlineStr">
         <is>
-          <t>Donair Sub</t>
+          <t>Pizza Sub</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr"/>
       <c r="E108" s="10" t="n">
-        <v>11.95</v>
+        <v>10.95</v>
       </c>
       <c r="F108" s="10" t="n">
-        <v>14.95</v>
+        <v>13.25</v>
       </c>
       <c r="G108" s="10" t="n"/>
       <c r="H108" s="10" t="n"/>
@@ -4736,7 +4692,7 @@
     <row r="109">
       <c r="A109" s="9" t="inlineStr">
         <is>
-          <t>subs/Super Sub</t>
+          <t>subs/Vegetarian</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
@@ -4746,15 +4702,15 @@
       </c>
       <c r="C109" s="10" t="inlineStr">
         <is>
-          <t>Super Sub</t>
+          <t>Vegetarian</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr"/>
       <c r="E109" s="10" t="n">
-        <v>12.45</v>
+        <v>10.95</v>
       </c>
       <c r="F109" s="10" t="n">
-        <v>16.25</v>
+        <v>13.25</v>
       </c>
       <c r="G109" s="10" t="n"/>
       <c r="H109" s="10" t="n"/>
@@ -4768,7 +4724,7 @@
     <row r="110">
       <c r="A110" s="9" t="inlineStr">
         <is>
-          <t>subs/Garlic Bread</t>
+          <t>subs/Real Turkey</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
@@ -4778,15 +4734,15 @@
       </c>
       <c r="C110" s="10" t="inlineStr">
         <is>
-          <t>Garlic Bread</t>
+          <t>Real Turkey</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr"/>
       <c r="E110" s="10" t="n">
-        <v>6.25</v>
+        <v>11.45</v>
       </c>
       <c r="F110" s="10" t="n">
-        <v>7.45</v>
+        <v>13.25</v>
       </c>
       <c r="G110" s="10" t="n"/>
       <c r="H110" s="10" t="n"/>
@@ -4800,7 +4756,7 @@
     <row r="111">
       <c r="A111" s="9" t="inlineStr">
         <is>
-          <t>subs/Extra Cheese</t>
+          <t>subs/Bubba</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
@@ -4810,15 +4766,19 @@
       </c>
       <c r="C111" s="10" t="inlineStr">
         <is>
-          <t>Extra Cheese</t>
-        </is>
-      </c>
-      <c r="D111" s="10" t="inlineStr"/>
+          <t>Bubba</t>
+        </is>
+      </c>
+      <c r="D111" s="10" t="inlineStr">
+        <is>
+          <t>The one people ask for by name.</t>
+        </is>
+      </c>
       <c r="E111" s="10" t="n">
-        <v>2.75</v>
+        <v>11.95</v>
       </c>
       <c r="F111" s="10" t="n">
-        <v>3.95</v>
+        <v>14.25</v>
       </c>
       <c r="G111" s="10" t="n"/>
       <c r="H111" s="10" t="n"/>
@@ -4832,7 +4792,7 @@
     <row r="112">
       <c r="A112" s="9" t="inlineStr">
         <is>
-          <t>subs/Extra Meat</t>
+          <t>subs/Club</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
@@ -4842,15 +4802,15 @@
       </c>
       <c r="C112" s="10" t="inlineStr">
         <is>
-          <t>Extra Meat</t>
+          <t>Club</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr"/>
       <c r="E112" s="10" t="n">
-        <v>3.95</v>
+        <v>11.95</v>
       </c>
       <c r="F112" s="10" t="n">
-        <v>4.75</v>
+        <v>14.25</v>
       </c>
       <c r="G112" s="10" t="n"/>
       <c r="H112" s="10" t="n"/>
@@ -4864,105 +4824,99 @@
     <row r="113">
       <c r="A113" s="9" t="inlineStr">
         <is>
-          <t>burritos/Beans &amp; Veggie</t>
+          <t>subs/Steak</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
         <is>
-          <t>Burritos</t>
+          <t>Subs</t>
         </is>
       </c>
       <c r="C113" s="10" t="inlineStr">
         <is>
-          <t>Beans &amp; Veggie</t>
+          <t>Steak</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr"/>
       <c r="E113" s="10" t="n">
-        <v>7.99</v>
+        <v>11.95</v>
       </c>
       <c r="F113" s="10" t="n">
-        <v>8.99</v>
-      </c>
-      <c r="G113" s="10" t="n">
-        <v>10.99</v>
-      </c>
+        <v>14.95</v>
+      </c>
+      <c r="G113" s="10" t="n"/>
       <c r="H113" s="10" t="n"/>
       <c r="I113" s="10" t="inlineStr">
         <is>
-          <t>Small / Medium / Large</t>
-        </is>
-      </c>
-      <c r="J113" s="10" t="inlineStr"/>
+          <t>Small / Large</t>
+        </is>
+      </c>
+      <c r="J113" s="10" t="inlineStr">
+        <is>
+          <t>steak-sub</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="9" t="inlineStr">
         <is>
-          <t>burritos/Spicy Chicken</t>
+          <t>subs/Donair Sub</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
         <is>
-          <t>Burritos</t>
+          <t>Subs</t>
         </is>
       </c>
       <c r="C114" s="10" t="inlineStr">
         <is>
-          <t>Spicy Chicken</t>
+          <t>Donair Sub</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr"/>
       <c r="E114" s="10" t="n">
-        <v>9.99</v>
+        <v>11.95</v>
       </c>
       <c r="F114" s="10" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G114" s="10" t="n">
-        <v>12.99</v>
-      </c>
+        <v>14.95</v>
+      </c>
+      <c r="G114" s="10" t="n"/>
       <c r="H114" s="10" t="n"/>
       <c r="I114" s="10" t="inlineStr">
         <is>
-          <t>Small / Medium / Large</t>
-        </is>
-      </c>
-      <c r="J114" s="10" t="inlineStr">
-        <is>
-          <t>burrito</t>
-        </is>
-      </c>
+          <t>Small / Large</t>
+        </is>
+      </c>
+      <c r="J114" s="10" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>burritos/Ground Beef</t>
+          <t>subs/Super Sub</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
         <is>
-          <t>Burritos</t>
+          <t>Subs</t>
         </is>
       </c>
       <c r="C115" s="10" t="inlineStr">
         <is>
-          <t>Ground Beef</t>
+          <t>Super Sub</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr"/>
       <c r="E115" s="10" t="n">
-        <v>9.99</v>
+        <v>12.45</v>
       </c>
       <c r="F115" s="10" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G115" s="10" t="n">
-        <v>12.99</v>
-      </c>
+        <v>16.25</v>
+      </c>
+      <c r="G115" s="10" t="n"/>
       <c r="H115" s="10" t="n"/>
       <c r="I115" s="10" t="inlineStr">
         <is>
-          <t>Small / Medium / Large</t>
+          <t>Small / Large</t>
         </is>
       </c>
       <c r="J115" s="10" t="inlineStr"/>
@@ -4970,33 +4924,31 @@
     <row r="116">
       <c r="A116" s="9" t="inlineStr">
         <is>
-          <t>burritos/Zesty Grilled Chicken</t>
+          <t>subs/Garlic Bread</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
         <is>
-          <t>Burritos</t>
+          <t>Subs</t>
         </is>
       </c>
       <c r="C116" s="10" t="inlineStr">
         <is>
-          <t>Zesty Grilled Chicken</t>
+          <t>Garlic Bread</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr"/>
       <c r="E116" s="10" t="n">
-        <v>9.99</v>
+        <v>6.25</v>
       </c>
       <c r="F116" s="10" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G116" s="10" t="n">
-        <v>12.99</v>
-      </c>
+        <v>7.45</v>
+      </c>
+      <c r="G116" s="10" t="n"/>
       <c r="H116" s="10" t="n"/>
       <c r="I116" s="10" t="inlineStr">
         <is>
-          <t>Small / Medium / Large</t>
+          <t>Small / Large</t>
         </is>
       </c>
       <c r="J116" s="10" t="inlineStr"/>
@@ -5004,33 +4956,31 @@
     <row r="117">
       <c r="A117" s="9" t="inlineStr">
         <is>
-          <t>burritos/Fish</t>
+          <t>subs/Extra Cheese</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
         <is>
-          <t>Burritos</t>
+          <t>Subs</t>
         </is>
       </c>
       <c r="C117" s="10" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Extra Cheese</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr"/>
       <c r="E117" s="10" t="n">
-        <v>9.99</v>
+        <v>2.75</v>
       </c>
       <c r="F117" s="10" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G117" s="10" t="n">
-        <v>12.99</v>
-      </c>
+        <v>3.95</v>
+      </c>
+      <c r="G117" s="10" t="n"/>
       <c r="H117" s="10" t="n"/>
       <c r="I117" s="10" t="inlineStr">
         <is>
-          <t>Small / Medium / Large</t>
+          <t>Small / Large</t>
         </is>
       </c>
       <c r="J117" s="10" t="inlineStr"/>
@@ -5038,33 +4988,31 @@
     <row r="118">
       <c r="A118" s="9" t="inlineStr">
         <is>
-          <t>burritos/Shawarma Chicken</t>
+          <t>subs/Extra Meat</t>
         </is>
       </c>
       <c r="B118" s="10" t="inlineStr">
         <is>
-          <t>Burritos</t>
+          <t>Subs</t>
         </is>
       </c>
       <c r="C118" s="10" t="inlineStr">
         <is>
-          <t>Shawarma Chicken</t>
+          <t>Extra Meat</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr"/>
       <c r="E118" s="10" t="n">
-        <v>10.99</v>
+        <v>3.95</v>
       </c>
       <c r="F118" s="10" t="n">
-        <v>11.99</v>
-      </c>
-      <c r="G118" s="10" t="n">
-        <v>13.99</v>
-      </c>
+        <v>4.75</v>
+      </c>
+      <c r="G118" s="10" t="n"/>
       <c r="H118" s="10" t="n"/>
       <c r="I118" s="10" t="inlineStr">
         <is>
-          <t>Small / Medium / Large</t>
+          <t>Small / Large</t>
         </is>
       </c>
       <c r="J118" s="10" t="inlineStr"/>
@@ -5072,7 +5020,7 @@
     <row r="119">
       <c r="A119" s="9" t="inlineStr">
         <is>
-          <t>burritos/Tequila-Lime Glazed Chicken</t>
+          <t>burritos/Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="B119" s="10" t="inlineStr">
@@ -5082,18 +5030,18 @@
       </c>
       <c r="C119" s="10" t="inlineStr">
         <is>
-          <t>Tequila-Lime Glazed Chicken</t>
+          <t>Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr"/>
       <c r="E119" s="10" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="F119" s="10" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="G119" s="10" t="n">
         <v>10.99</v>
-      </c>
-      <c r="F119" s="10" t="n">
-        <v>11.99</v>
-      </c>
-      <c r="G119" s="10" t="n">
-        <v>13.99</v>
       </c>
       <c r="H119" s="10" t="n"/>
       <c r="I119" s="10" t="inlineStr">
@@ -5106,7 +5054,7 @@
     <row r="120">
       <c r="A120" s="9" t="inlineStr">
         <is>
-          <t>burritos/Steak</t>
+          <t>burritos/Spicy Chicken</t>
         </is>
       </c>
       <c r="B120" s="10" t="inlineStr">
@@ -5116,18 +5064,18 @@
       </c>
       <c r="C120" s="10" t="inlineStr">
         <is>
-          <t>Steak</t>
+          <t>Spicy Chicken</t>
         </is>
       </c>
       <c r="D120" s="10" t="inlineStr"/>
       <c r="E120" s="10" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="F120" s="10" t="n">
         <v>10.99</v>
       </c>
-      <c r="F120" s="10" t="n">
-        <v>11.99</v>
-      </c>
       <c r="G120" s="10" t="n">
-        <v>13.99</v>
+        <v>12.99</v>
       </c>
       <c r="H120" s="10" t="n"/>
       <c r="I120" s="10" t="inlineStr">
@@ -5135,72 +5083,76 @@
           <t>Small / Medium / Large</t>
         </is>
       </c>
-      <c r="J120" s="10" t="inlineStr"/>
+      <c r="J120" s="10" t="inlineStr">
+        <is>
+          <t>burrito</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Beans &amp; Veggie</t>
+          <t>burritos/Ground Beef</t>
         </is>
       </c>
       <c r="B121" s="10" t="inlineStr">
         <is>
-          <t>Rice Bowls</t>
+          <t>Burritos</t>
         </is>
       </c>
       <c r="C121" s="10" t="inlineStr">
         <is>
-          <t>Beans &amp; Veggie</t>
+          <t>Ground Beef</t>
         </is>
       </c>
       <c r="D121" s="10" t="inlineStr"/>
       <c r="E121" s="10" t="n">
-        <v>10.49</v>
+        <v>9.99</v>
       </c>
       <c r="F121" s="10" t="n">
-        <v>12.49</v>
-      </c>
-      <c r="G121" s="10" t="n"/>
+        <v>10.99</v>
+      </c>
+      <c r="G121" s="10" t="n">
+        <v>12.99</v>
+      </c>
       <c r="H121" s="10" t="n"/>
       <c r="I121" s="10" t="inlineStr">
         <is>
-          <t>Small / Large</t>
-        </is>
-      </c>
-      <c r="J121" s="10" t="inlineStr">
-        <is>
-          <t>rice-bowl</t>
-        </is>
-      </c>
+          <t>Small / Medium / Large</t>
+        </is>
+      </c>
+      <c r="J121" s="10" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Spicy Chicken</t>
+          <t>burritos/Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="B122" s="10" t="inlineStr">
         <is>
-          <t>Rice Bowls</t>
+          <t>Burritos</t>
         </is>
       </c>
       <c r="C122" s="10" t="inlineStr">
         <is>
-          <t>Spicy Chicken</t>
+          <t>Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr"/>
       <c r="E122" s="10" t="n">
-        <v>11.49</v>
+        <v>9.99</v>
       </c>
       <c r="F122" s="10" t="n">
-        <v>13.49</v>
-      </c>
-      <c r="G122" s="10" t="n"/>
+        <v>10.99</v>
+      </c>
+      <c r="G122" s="10" t="n">
+        <v>12.99</v>
+      </c>
       <c r="H122" s="10" t="n"/>
       <c r="I122" s="10" t="inlineStr">
         <is>
-          <t>Small / Large</t>
+          <t>Small / Medium / Large</t>
         </is>
       </c>
       <c r="J122" s="10" t="inlineStr"/>
@@ -5208,31 +5160,33 @@
     <row r="123">
       <c r="A123" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Ground Beef</t>
+          <t>burritos/Fish</t>
         </is>
       </c>
       <c r="B123" s="10" t="inlineStr">
         <is>
-          <t>Rice Bowls</t>
+          <t>Burritos</t>
         </is>
       </c>
       <c r="C123" s="10" t="inlineStr">
         <is>
-          <t>Ground Beef</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D123" s="10" t="inlineStr"/>
       <c r="E123" s="10" t="n">
-        <v>11.49</v>
+        <v>9.99</v>
       </c>
       <c r="F123" s="10" t="n">
-        <v>13.49</v>
-      </c>
-      <c r="G123" s="10" t="n"/>
+        <v>10.99</v>
+      </c>
+      <c r="G123" s="10" t="n">
+        <v>12.99</v>
+      </c>
       <c r="H123" s="10" t="n"/>
       <c r="I123" s="10" t="inlineStr">
         <is>
-          <t>Small / Large</t>
+          <t>Small / Medium / Large</t>
         </is>
       </c>
       <c r="J123" s="10" t="inlineStr"/>
@@ -5240,31 +5194,33 @@
     <row r="124">
       <c r="A124" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Zesty Grilled Chicken</t>
+          <t>burritos/Shawarma Chicken</t>
         </is>
       </c>
       <c r="B124" s="10" t="inlineStr">
         <is>
-          <t>Rice Bowls</t>
+          <t>Burritos</t>
         </is>
       </c>
       <c r="C124" s="10" t="inlineStr">
         <is>
-          <t>Zesty Grilled Chicken</t>
+          <t>Shawarma Chicken</t>
         </is>
       </c>
       <c r="D124" s="10" t="inlineStr"/>
       <c r="E124" s="10" t="n">
-        <v>11.49</v>
+        <v>10.99</v>
       </c>
       <c r="F124" s="10" t="n">
-        <v>13.49</v>
-      </c>
-      <c r="G124" s="10" t="n"/>
+        <v>11.99</v>
+      </c>
+      <c r="G124" s="10" t="n">
+        <v>13.99</v>
+      </c>
       <c r="H124" s="10" t="n"/>
       <c r="I124" s="10" t="inlineStr">
         <is>
-          <t>Small / Large</t>
+          <t>Small / Medium / Large</t>
         </is>
       </c>
       <c r="J124" s="10" t="inlineStr"/>
@@ -5272,31 +5228,33 @@
     <row r="125">
       <c r="A125" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Fish</t>
+          <t>burritos/Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="B125" s="10" t="inlineStr">
         <is>
-          <t>Rice Bowls</t>
+          <t>Burritos</t>
         </is>
       </c>
       <c r="C125" s="10" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr"/>
       <c r="E125" s="10" t="n">
-        <v>11.49</v>
+        <v>10.99</v>
       </c>
       <c r="F125" s="10" t="n">
-        <v>13.49</v>
-      </c>
-      <c r="G125" s="10" t="n"/>
+        <v>11.99</v>
+      </c>
+      <c r="G125" s="10" t="n">
+        <v>13.99</v>
+      </c>
       <c r="H125" s="10" t="n"/>
       <c r="I125" s="10" t="inlineStr">
         <is>
-          <t>Small / Large</t>
+          <t>Small / Medium / Large</t>
         </is>
       </c>
       <c r="J125" s="10" t="inlineStr"/>
@@ -5304,31 +5262,33 @@
     <row r="126">
       <c r="A126" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Shawarma Chicken</t>
+          <t>burritos/Steak</t>
         </is>
       </c>
       <c r="B126" s="10" t="inlineStr">
         <is>
-          <t>Rice Bowls</t>
+          <t>Burritos</t>
         </is>
       </c>
       <c r="C126" s="10" t="inlineStr">
         <is>
-          <t>Shawarma Chicken</t>
+          <t>Steak</t>
         </is>
       </c>
       <c r="D126" s="10" t="inlineStr"/>
       <c r="E126" s="10" t="n">
-        <v>12.49</v>
+        <v>10.99</v>
       </c>
       <c r="F126" s="10" t="n">
-        <v>14.49</v>
-      </c>
-      <c r="G126" s="10" t="n"/>
+        <v>11.99</v>
+      </c>
+      <c r="G126" s="10" t="n">
+        <v>13.99</v>
+      </c>
       <c r="H126" s="10" t="n"/>
       <c r="I126" s="10" t="inlineStr">
         <is>
-          <t>Small / Large</t>
+          <t>Small / Medium / Large</t>
         </is>
       </c>
       <c r="J126" s="10" t="inlineStr"/>
@@ -5336,7 +5296,7 @@
     <row r="127">
       <c r="A127" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Tequila-Lime Glazed Chicken</t>
+          <t>rice-bowls/Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="B127" s="10" t="inlineStr">
@@ -5346,15 +5306,15 @@
       </c>
       <c r="C127" s="10" t="inlineStr">
         <is>
-          <t>Tequila-Lime Glazed Chicken</t>
+          <t>Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="D127" s="10" t="inlineStr"/>
       <c r="E127" s="10" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="F127" s="10" t="n">
         <v>12.49</v>
-      </c>
-      <c r="F127" s="10" t="n">
-        <v>14.49</v>
       </c>
       <c r="G127" s="10" t="n"/>
       <c r="H127" s="10" t="n"/>
@@ -5363,12 +5323,16 @@
           <t>Small / Large</t>
         </is>
       </c>
-      <c r="J127" s="10" t="inlineStr"/>
+      <c r="J127" s="10" t="inlineStr">
+        <is>
+          <t>rice-bowl</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Steak</t>
+          <t>rice-bowls/Spicy Chicken</t>
         </is>
       </c>
       <c r="B128" s="10" t="inlineStr">
@@ -5378,15 +5342,15 @@
       </c>
       <c r="C128" s="10" t="inlineStr">
         <is>
-          <t>Steak</t>
+          <t>Spicy Chicken</t>
         </is>
       </c>
       <c r="D128" s="10" t="inlineStr"/>
       <c r="E128" s="10" t="n">
-        <v>12.49</v>
+        <v>11.49</v>
       </c>
       <c r="F128" s="10" t="n">
-        <v>14.49</v>
+        <v>13.49</v>
       </c>
       <c r="G128" s="10" t="n"/>
       <c r="H128" s="10" t="n"/>
@@ -5400,167 +5364,199 @@
     <row r="129">
       <c r="A129" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Beans &amp; Veggie</t>
+          <t>rice-bowls/Ground Beef</t>
         </is>
       </c>
       <c r="B129" s="10" t="inlineStr">
         <is>
-          <t>Quesadillas</t>
+          <t>Rice Bowls</t>
         </is>
       </c>
       <c r="C129" s="10" t="inlineStr">
         <is>
-          <t>Beans &amp; Veggie</t>
+          <t>Ground Beef</t>
         </is>
       </c>
       <c r="D129" s="10" t="inlineStr"/>
       <c r="E129" s="10" t="n">
-        <v>10.49</v>
-      </c>
-      <c r="F129" s="10" t="n"/>
+        <v>11.49</v>
+      </c>
+      <c r="F129" s="10" t="n">
+        <v>13.49</v>
+      </c>
       <c r="G129" s="10" t="n"/>
       <c r="H129" s="10" t="n"/>
-      <c r="I129" s="10" t="inlineStr"/>
-      <c r="J129" s="10" t="inlineStr">
-        <is>
-          <t>quesadilla</t>
-        </is>
-      </c>
+      <c r="I129" s="10" t="inlineStr">
+        <is>
+          <t>Small / Large</t>
+        </is>
+      </c>
+      <c r="J129" s="10" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Spicy Chicken</t>
+          <t>rice-bowls/Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="B130" s="10" t="inlineStr">
         <is>
-          <t>Quesadillas</t>
+          <t>Rice Bowls</t>
         </is>
       </c>
       <c r="C130" s="10" t="inlineStr">
         <is>
-          <t>Spicy Chicken</t>
+          <t>Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="D130" s="10" t="inlineStr"/>
       <c r="E130" s="10" t="n">
         <v>11.49</v>
       </c>
-      <c r="F130" s="10" t="n"/>
+      <c r="F130" s="10" t="n">
+        <v>13.49</v>
+      </c>
       <c r="G130" s="10" t="n"/>
       <c r="H130" s="10" t="n"/>
-      <c r="I130" s="10" t="inlineStr"/>
+      <c r="I130" s="10" t="inlineStr">
+        <is>
+          <t>Small / Large</t>
+        </is>
+      </c>
       <c r="J130" s="10" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Ground Beef</t>
+          <t>rice-bowls/Fish</t>
         </is>
       </c>
       <c r="B131" s="10" t="inlineStr">
         <is>
-          <t>Quesadillas</t>
+          <t>Rice Bowls</t>
         </is>
       </c>
       <c r="C131" s="10" t="inlineStr">
         <is>
-          <t>Ground Beef</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D131" s="10" t="inlineStr"/>
       <c r="E131" s="10" t="n">
         <v>11.49</v>
       </c>
-      <c r="F131" s="10" t="n"/>
+      <c r="F131" s="10" t="n">
+        <v>13.49</v>
+      </c>
       <c r="G131" s="10" t="n"/>
       <c r="H131" s="10" t="n"/>
-      <c r="I131" s="10" t="inlineStr"/>
+      <c r="I131" s="10" t="inlineStr">
+        <is>
+          <t>Small / Large</t>
+        </is>
+      </c>
       <c r="J131" s="10" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Zesty Grilled Chicken</t>
+          <t>rice-bowls/Shawarma Chicken</t>
         </is>
       </c>
       <c r="B132" s="10" t="inlineStr">
         <is>
-          <t>Quesadillas</t>
+          <t>Rice Bowls</t>
         </is>
       </c>
       <c r="C132" s="10" t="inlineStr">
         <is>
-          <t>Zesty Grilled Chicken</t>
+          <t>Shawarma Chicken</t>
         </is>
       </c>
       <c r="D132" s="10" t="inlineStr"/>
       <c r="E132" s="10" t="n">
-        <v>11.49</v>
-      </c>
-      <c r="F132" s="10" t="n"/>
+        <v>12.49</v>
+      </c>
+      <c r="F132" s="10" t="n">
+        <v>14.49</v>
+      </c>
       <c r="G132" s="10" t="n"/>
       <c r="H132" s="10" t="n"/>
-      <c r="I132" s="10" t="inlineStr"/>
+      <c r="I132" s="10" t="inlineStr">
+        <is>
+          <t>Small / Large</t>
+        </is>
+      </c>
       <c r="J132" s="10" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Fish</t>
+          <t>rice-bowls/Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="B133" s="10" t="inlineStr">
         <is>
-          <t>Quesadillas</t>
+          <t>Rice Bowls</t>
         </is>
       </c>
       <c r="C133" s="10" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="D133" s="10" t="inlineStr"/>
       <c r="E133" s="10" t="n">
-        <v>11.49</v>
-      </c>
-      <c r="F133" s="10" t="n"/>
+        <v>12.49</v>
+      </c>
+      <c r="F133" s="10" t="n">
+        <v>14.49</v>
+      </c>
       <c r="G133" s="10" t="n"/>
       <c r="H133" s="10" t="n"/>
-      <c r="I133" s="10" t="inlineStr"/>
+      <c r="I133" s="10" t="inlineStr">
+        <is>
+          <t>Small / Large</t>
+        </is>
+      </c>
       <c r="J133" s="10" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Shawarma Chicken</t>
+          <t>rice-bowls/Steak</t>
         </is>
       </c>
       <c r="B134" s="10" t="inlineStr">
         <is>
-          <t>Quesadillas</t>
+          <t>Rice Bowls</t>
         </is>
       </c>
       <c r="C134" s="10" t="inlineStr">
         <is>
-          <t>Shawarma Chicken</t>
+          <t>Steak</t>
         </is>
       </c>
       <c r="D134" s="10" t="inlineStr"/>
       <c r="E134" s="10" t="n">
         <v>12.49</v>
       </c>
-      <c r="F134" s="10" t="n"/>
+      <c r="F134" s="10" t="n">
+        <v>14.49</v>
+      </c>
       <c r="G134" s="10" t="n"/>
       <c r="H134" s="10" t="n"/>
-      <c r="I134" s="10" t="inlineStr"/>
+      <c r="I134" s="10" t="inlineStr">
+        <is>
+          <t>Small / Large</t>
+        </is>
+      </c>
       <c r="J134" s="10" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Tequila-Lime Glazed Chicken</t>
+          <t>quesadillas/Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="B135" s="10" t="inlineStr">
@@ -5570,23 +5566,27 @@
       </c>
       <c r="C135" s="10" t="inlineStr">
         <is>
-          <t>Tequila-Lime Glazed Chicken</t>
+          <t>Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="D135" s="10" t="inlineStr"/>
       <c r="E135" s="10" t="n">
-        <v>12.49</v>
+        <v>10.49</v>
       </c>
       <c r="F135" s="10" t="n"/>
       <c r="G135" s="10" t="n"/>
       <c r="H135" s="10" t="n"/>
       <c r="I135" s="10" t="inlineStr"/>
-      <c r="J135" s="10" t="inlineStr"/>
+      <c r="J135" s="10" t="inlineStr">
+        <is>
+          <t>quesadilla</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Steak</t>
+          <t>quesadillas/Spicy Chicken</t>
         </is>
       </c>
       <c r="B136" s="10" t="inlineStr">
@@ -5596,12 +5596,12 @@
       </c>
       <c r="C136" s="10" t="inlineStr">
         <is>
-          <t>Steak</t>
+          <t>Spicy Chicken</t>
         </is>
       </c>
       <c r="D136" s="10" t="inlineStr"/>
       <c r="E136" s="10" t="n">
-        <v>12.49</v>
+        <v>11.49</v>
       </c>
       <c r="F136" s="10" t="n"/>
       <c r="G136" s="10" t="n"/>
@@ -5612,52 +5612,48 @@
     <row r="137">
       <c r="A137" s="9" t="inlineStr">
         <is>
-          <t>tacos/Beans &amp; Veggie</t>
+          <t>quesadillas/Ground Beef</t>
         </is>
       </c>
       <c r="B137" s="10" t="inlineStr">
         <is>
-          <t>Tacos</t>
+          <t>Quesadillas</t>
         </is>
       </c>
       <c r="C137" s="10" t="inlineStr">
         <is>
-          <t>Beans &amp; Veggie</t>
+          <t>Ground Beef</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr"/>
       <c r="E137" s="10" t="n">
-        <v>9.99</v>
+        <v>11.49</v>
       </c>
       <c r="F137" s="10" t="n"/>
       <c r="G137" s="10" t="n"/>
       <c r="H137" s="10" t="n"/>
       <c r="I137" s="10" t="inlineStr"/>
-      <c r="J137" s="10" t="inlineStr">
-        <is>
-          <t>tacos</t>
-        </is>
-      </c>
+      <c r="J137" s="10" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="9" t="inlineStr">
         <is>
-          <t>tacos/Spicy Chicken</t>
+          <t>quesadillas/Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="B138" s="10" t="inlineStr">
         <is>
-          <t>Tacos</t>
+          <t>Quesadillas</t>
         </is>
       </c>
       <c r="C138" s="10" t="inlineStr">
         <is>
-          <t>Spicy Chicken</t>
+          <t>Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="D138" s="10" t="inlineStr"/>
       <c r="E138" s="10" t="n">
-        <v>10.99</v>
+        <v>11.49</v>
       </c>
       <c r="F138" s="10" t="n"/>
       <c r="G138" s="10" t="n"/>
@@ -5668,22 +5664,22 @@
     <row r="139">
       <c r="A139" s="9" t="inlineStr">
         <is>
-          <t>tacos/Ground Beef</t>
+          <t>quesadillas/Fish</t>
         </is>
       </c>
       <c r="B139" s="10" t="inlineStr">
         <is>
-          <t>Tacos</t>
+          <t>Quesadillas</t>
         </is>
       </c>
       <c r="C139" s="10" t="inlineStr">
         <is>
-          <t>Ground Beef</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D139" s="10" t="inlineStr"/>
       <c r="E139" s="10" t="n">
-        <v>10.99</v>
+        <v>11.49</v>
       </c>
       <c r="F139" s="10" t="n"/>
       <c r="G139" s="10" t="n"/>
@@ -5694,22 +5690,22 @@
     <row r="140">
       <c r="A140" s="9" t="inlineStr">
         <is>
-          <t>tacos/Zesty Grilled Chicken</t>
+          <t>quesadillas/Shawarma Chicken</t>
         </is>
       </c>
       <c r="B140" s="10" t="inlineStr">
         <is>
-          <t>Tacos</t>
+          <t>Quesadillas</t>
         </is>
       </c>
       <c r="C140" s="10" t="inlineStr">
         <is>
-          <t>Zesty Grilled Chicken</t>
+          <t>Shawarma Chicken</t>
         </is>
       </c>
       <c r="D140" s="10" t="inlineStr"/>
       <c r="E140" s="10" t="n">
-        <v>10.99</v>
+        <v>12.49</v>
       </c>
       <c r="F140" s="10" t="n"/>
       <c r="G140" s="10" t="n"/>
@@ -5720,22 +5716,22 @@
     <row r="141">
       <c r="A141" s="9" t="inlineStr">
         <is>
-          <t>tacos/Fish</t>
+          <t>quesadillas/Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="B141" s="10" t="inlineStr">
         <is>
-          <t>Tacos</t>
+          <t>Quesadillas</t>
         </is>
       </c>
       <c r="C141" s="10" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="D141" s="10" t="inlineStr"/>
       <c r="E141" s="10" t="n">
-        <v>10.99</v>
+        <v>12.49</v>
       </c>
       <c r="F141" s="10" t="n"/>
       <c r="G141" s="10" t="n"/>
@@ -5746,22 +5742,22 @@
     <row r="142">
       <c r="A142" s="9" t="inlineStr">
         <is>
-          <t>tacos/Shawarma Chicken</t>
+          <t>quesadillas/Steak</t>
         </is>
       </c>
       <c r="B142" s="10" t="inlineStr">
         <is>
-          <t>Tacos</t>
+          <t>Quesadillas</t>
         </is>
       </c>
       <c r="C142" s="10" t="inlineStr">
         <is>
-          <t>Shawarma Chicken</t>
+          <t>Steak</t>
         </is>
       </c>
       <c r="D142" s="10" t="inlineStr"/>
       <c r="E142" s="10" t="n">
-        <v>11.99</v>
+        <v>12.49</v>
       </c>
       <c r="F142" s="10" t="n"/>
       <c r="G142" s="10" t="n"/>
@@ -5772,7 +5768,7 @@
     <row r="143">
       <c r="A143" s="9" t="inlineStr">
         <is>
-          <t>tacos/Tequila-Lime Glazed Chicken</t>
+          <t>tacos/Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="B143" s="10" t="inlineStr">
@@ -5782,23 +5778,27 @@
       </c>
       <c r="C143" s="10" t="inlineStr">
         <is>
-          <t>Tequila-Lime Glazed Chicken</t>
+          <t>Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="D143" s="10" t="inlineStr"/>
       <c r="E143" s="10" t="n">
-        <v>11.99</v>
+        <v>9.99</v>
       </c>
       <c r="F143" s="10" t="n"/>
       <c r="G143" s="10" t="n"/>
       <c r="H143" s="10" t="n"/>
       <c r="I143" s="10" t="inlineStr"/>
-      <c r="J143" s="10" t="inlineStr"/>
+      <c r="J143" s="10" t="inlineStr">
+        <is>
+          <t>tacos</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="9" t="inlineStr">
         <is>
-          <t>tacos/Steak</t>
+          <t>tacos/Spicy Chicken</t>
         </is>
       </c>
       <c r="B144" s="10" t="inlineStr">
@@ -5808,12 +5808,12 @@
       </c>
       <c r="C144" s="10" t="inlineStr">
         <is>
-          <t>Steak</t>
+          <t>Spicy Chicken</t>
         </is>
       </c>
       <c r="D144" s="10" t="inlineStr"/>
       <c r="E144" s="10" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="F144" s="10" t="n"/>
       <c r="G144" s="10" t="n"/>
@@ -5824,22 +5824,22 @@
     <row r="145">
       <c r="A145" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Chips &amp; Salsa — Small</t>
+          <t>tacos/Ground Beef</t>
         </is>
       </c>
       <c r="B145" s="10" t="inlineStr">
         <is>
-          <t>Sides</t>
+          <t>Tacos</t>
         </is>
       </c>
       <c r="C145" s="10" t="inlineStr">
         <is>
-          <t>Chips &amp; Salsa — Small</t>
+          <t>Ground Beef</t>
         </is>
       </c>
       <c r="D145" s="10" t="inlineStr"/>
       <c r="E145" s="10" t="n">
-        <v>2.49</v>
+        <v>10.99</v>
       </c>
       <c r="F145" s="10" t="n"/>
       <c r="G145" s="10" t="n"/>
@@ -5850,22 +5850,22 @@
     <row r="146">
       <c r="A146" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Chips &amp; Salsa — Large</t>
+          <t>tacos/Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="B146" s="10" t="inlineStr">
         <is>
-          <t>Sides</t>
+          <t>Tacos</t>
         </is>
       </c>
       <c r="C146" s="10" t="inlineStr">
         <is>
-          <t>Chips &amp; Salsa — Large</t>
+          <t>Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="D146" s="10" t="inlineStr"/>
       <c r="E146" s="10" t="n">
-        <v>4.49</v>
+        <v>10.99</v>
       </c>
       <c r="F146" s="10" t="n"/>
       <c r="G146" s="10" t="n"/>
@@ -5876,22 +5876,22 @@
     <row r="147">
       <c r="A147" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Chips &amp; Queso — Small</t>
+          <t>tacos/Fish</t>
         </is>
       </c>
       <c r="B147" s="10" t="inlineStr">
         <is>
-          <t>Sides</t>
+          <t>Tacos</t>
         </is>
       </c>
       <c r="C147" s="10" t="inlineStr">
         <is>
-          <t>Chips &amp; Queso — Small</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D147" s="10" t="inlineStr"/>
       <c r="E147" s="10" t="n">
-        <v>3.49</v>
+        <v>10.99</v>
       </c>
       <c r="F147" s="10" t="n"/>
       <c r="G147" s="10" t="n"/>
@@ -5902,22 +5902,22 @@
     <row r="148">
       <c r="A148" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Chips &amp; Queso — Large</t>
+          <t>tacos/Shawarma Chicken</t>
         </is>
       </c>
       <c r="B148" s="10" t="inlineStr">
         <is>
-          <t>Sides</t>
+          <t>Tacos</t>
         </is>
       </c>
       <c r="C148" s="10" t="inlineStr">
         <is>
-          <t>Chips &amp; Queso — Large</t>
+          <t>Shawarma Chicken</t>
         </is>
       </c>
       <c r="D148" s="10" t="inlineStr"/>
       <c r="E148" s="10" t="n">
-        <v>6.49</v>
+        <v>11.99</v>
       </c>
       <c r="F148" s="10" t="n"/>
       <c r="G148" s="10" t="n"/>
@@ -5928,22 +5928,22 @@
     <row r="149">
       <c r="A149" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Chips &amp; Guac — Small</t>
+          <t>tacos/Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="B149" s="10" t="inlineStr">
         <is>
-          <t>Sides</t>
+          <t>Tacos</t>
         </is>
       </c>
       <c r="C149" s="10" t="inlineStr">
         <is>
-          <t>Chips &amp; Guac — Small</t>
+          <t>Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="D149" s="10" t="inlineStr"/>
       <c r="E149" s="10" t="n">
-        <v>3.99</v>
+        <v>11.99</v>
       </c>
       <c r="F149" s="10" t="n"/>
       <c r="G149" s="10" t="n"/>
@@ -5954,22 +5954,22 @@
     <row r="150">
       <c r="A150" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Chips &amp; Guac — Large</t>
+          <t>tacos/Steak</t>
         </is>
       </c>
       <c r="B150" s="10" t="inlineStr">
         <is>
-          <t>Sides</t>
+          <t>Tacos</t>
         </is>
       </c>
       <c r="C150" s="10" t="inlineStr">
         <is>
-          <t>Chips &amp; Guac — Large</t>
+          <t>Steak</t>
         </is>
       </c>
       <c r="D150" s="10" t="inlineStr"/>
       <c r="E150" s="10" t="n">
-        <v>6.99</v>
+        <v>11.99</v>
       </c>
       <c r="F150" s="10" t="n"/>
       <c r="G150" s="10" t="n"/>
@@ -5980,7 +5980,7 @@
     <row r="151">
       <c r="A151" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Fries Supreme</t>
+          <t>burrito-sides/Chips &amp; Salsa — Small</t>
         </is>
       </c>
       <c r="B151" s="10" t="inlineStr">
@@ -5990,12 +5990,12 @@
       </c>
       <c r="C151" s="10" t="inlineStr">
         <is>
-          <t>Fries Supreme</t>
+          <t>Chips &amp; Salsa — Small</t>
         </is>
       </c>
       <c r="D151" s="10" t="inlineStr"/>
       <c r="E151" s="10" t="n">
-        <v>9.99</v>
+        <v>2.49</v>
       </c>
       <c r="F151" s="10" t="n"/>
       <c r="G151" s="10" t="n"/>
@@ -6006,7 +6006,7 @@
     <row r="152">
       <c r="A152" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Spicy Fries</t>
+          <t>burrito-sides/Chips &amp; Salsa — Large</t>
         </is>
       </c>
       <c r="B152" s="10" t="inlineStr">
@@ -6016,12 +6016,12 @@
       </c>
       <c r="C152" s="10" t="inlineStr">
         <is>
-          <t>Spicy Fries</t>
+          <t>Chips &amp; Salsa — Large</t>
         </is>
       </c>
       <c r="D152" s="10" t="inlineStr"/>
       <c r="E152" s="10" t="n">
-        <v>8.99</v>
+        <v>4.49</v>
       </c>
       <c r="F152" s="10" t="n"/>
       <c r="G152" s="10" t="n"/>
@@ -6032,7 +6032,7 @@
     <row r="153">
       <c r="A153" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Deep Fried Pepperoni</t>
+          <t>burrito-sides/Chips &amp; Queso — Small</t>
         </is>
       </c>
       <c r="B153" s="10" t="inlineStr">
@@ -6042,16 +6042,12 @@
       </c>
       <c r="C153" s="10" t="inlineStr">
         <is>
-          <t>Deep Fried Pepperoni</t>
-        </is>
-      </c>
-      <c r="D153" s="10" t="inlineStr">
-        <is>
-          <t>With honey mustard sauce.</t>
-        </is>
-      </c>
+          <t>Chips &amp; Queso — Small</t>
+        </is>
+      </c>
+      <c r="D153" s="10" t="inlineStr"/>
       <c r="E153" s="10" t="n">
-        <v>12.99</v>
+        <v>3.49</v>
       </c>
       <c r="F153" s="10" t="n"/>
       <c r="G153" s="10" t="n"/>
@@ -6062,7 +6058,7 @@
     <row r="154">
       <c r="A154" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Add Chips &amp; Salsa + a Can of Pop</t>
+          <t>burrito-sides/Chips &amp; Queso — Large</t>
         </is>
       </c>
       <c r="B154" s="10" t="inlineStr">
@@ -6072,12 +6068,12 @@
       </c>
       <c r="C154" s="10" t="inlineStr">
         <is>
-          <t>Add Chips &amp; Salsa + a Can of Pop</t>
+          <t>Chips &amp; Queso — Large</t>
         </is>
       </c>
       <c r="D154" s="10" t="inlineStr"/>
       <c r="E154" s="10" t="n">
-        <v>3.49</v>
+        <v>6.49</v>
       </c>
       <c r="F154" s="10" t="n"/>
       <c r="G154" s="10" t="n"/>
@@ -6088,7 +6084,7 @@
     <row r="155">
       <c r="A155" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Brownie</t>
+          <t>burrito-sides/Chips &amp; Guac — Small</t>
         </is>
       </c>
       <c r="B155" s="10" t="inlineStr">
@@ -6098,12 +6094,12 @@
       </c>
       <c r="C155" s="10" t="inlineStr">
         <is>
-          <t>Brownie</t>
+          <t>Chips &amp; Guac — Small</t>
         </is>
       </c>
       <c r="D155" s="10" t="inlineStr"/>
       <c r="E155" s="10" t="n">
-        <v>2.99</v>
+        <v>3.99</v>
       </c>
       <c r="F155" s="10" t="n"/>
       <c r="G155" s="10" t="n"/>
@@ -6111,12 +6107,172 @@
       <c r="I155" s="10" t="inlineStr"/>
       <c r="J155" s="10" t="inlineStr"/>
     </row>
+    <row r="156">
+      <c r="A156" s="9" t="inlineStr">
+        <is>
+          <t>burrito-sides/Chips &amp; Guac — Large</t>
+        </is>
+      </c>
+      <c r="B156" s="10" t="inlineStr">
+        <is>
+          <t>Sides</t>
+        </is>
+      </c>
+      <c r="C156" s="10" t="inlineStr">
+        <is>
+          <t>Chips &amp; Guac — Large</t>
+        </is>
+      </c>
+      <c r="D156" s="10" t="inlineStr"/>
+      <c r="E156" s="10" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="F156" s="10" t="n"/>
+      <c r="G156" s="10" t="n"/>
+      <c r="H156" s="10" t="n"/>
+      <c r="I156" s="10" t="inlineStr"/>
+      <c r="J156" s="10" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="9" t="inlineStr">
+        <is>
+          <t>burrito-sides/Fries Supreme</t>
+        </is>
+      </c>
+      <c r="B157" s="10" t="inlineStr">
+        <is>
+          <t>Sides</t>
+        </is>
+      </c>
+      <c r="C157" s="10" t="inlineStr">
+        <is>
+          <t>Fries Supreme</t>
+        </is>
+      </c>
+      <c r="D157" s="10" t="inlineStr"/>
+      <c r="E157" s="10" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="F157" s="10" t="n"/>
+      <c r="G157" s="10" t="n"/>
+      <c r="H157" s="10" t="n"/>
+      <c r="I157" s="10" t="inlineStr"/>
+      <c r="J157" s="10" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="9" t="inlineStr">
+        <is>
+          <t>burrito-sides/Spicy Fries</t>
+        </is>
+      </c>
+      <c r="B158" s="10" t="inlineStr">
+        <is>
+          <t>Sides</t>
+        </is>
+      </c>
+      <c r="C158" s="10" t="inlineStr">
+        <is>
+          <t>Spicy Fries</t>
+        </is>
+      </c>
+      <c r="D158" s="10" t="inlineStr"/>
+      <c r="E158" s="10" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F158" s="10" t="n"/>
+      <c r="G158" s="10" t="n"/>
+      <c r="H158" s="10" t="n"/>
+      <c r="I158" s="10" t="inlineStr"/>
+      <c r="J158" s="10" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="9" t="inlineStr">
+        <is>
+          <t>burrito-sides/Deep Fried Pepperoni</t>
+        </is>
+      </c>
+      <c r="B159" s="10" t="inlineStr">
+        <is>
+          <t>Sides</t>
+        </is>
+      </c>
+      <c r="C159" s="10" t="inlineStr">
+        <is>
+          <t>Deep Fried Pepperoni</t>
+        </is>
+      </c>
+      <c r="D159" s="10" t="inlineStr">
+        <is>
+          <t>With honey mustard sauce.</t>
+        </is>
+      </c>
+      <c r="E159" s="10" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="F159" s="10" t="n"/>
+      <c r="G159" s="10" t="n"/>
+      <c r="H159" s="10" t="n"/>
+      <c r="I159" s="10" t="inlineStr"/>
+      <c r="J159" s="10" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="9" t="inlineStr">
+        <is>
+          <t>burrito-sides/Add Chips &amp; Salsa + a Can of Pop</t>
+        </is>
+      </c>
+      <c r="B160" s="10" t="inlineStr">
+        <is>
+          <t>Sides</t>
+        </is>
+      </c>
+      <c r="C160" s="10" t="inlineStr">
+        <is>
+          <t>Add Chips &amp; Salsa + a Can of Pop</t>
+        </is>
+      </c>
+      <c r="D160" s="10" t="inlineStr"/>
+      <c r="E160" s="10" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="F160" s="10" t="n"/>
+      <c r="G160" s="10" t="n"/>
+      <c r="H160" s="10" t="n"/>
+      <c r="I160" s="10" t="inlineStr"/>
+      <c r="J160" s="10" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="9" t="inlineStr">
+        <is>
+          <t>burrito-sides/Brownie</t>
+        </is>
+      </c>
+      <c r="B161" s="10" t="inlineStr">
+        <is>
+          <t>Sides</t>
+        </is>
+      </c>
+      <c r="C161" s="10" t="inlineStr">
+        <is>
+          <t>Brownie</t>
+        </is>
+      </c>
+      <c r="D161" s="10" t="inlineStr"/>
+      <c r="E161" s="10" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F161" s="10" t="n"/>
+      <c r="G161" s="10" t="n"/>
+      <c r="H161" s="10" t="n"/>
+      <c r="I161" s="10" t="inlineStr"/>
+      <c r="J161" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J5:J155" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the list" error="Pick one from the dropdown, or leave it empty." type="list">
+    <dataValidation sqref="J5:J161" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the list" error="Pick one from the dropdown, or leave it empty." type="list">
       <formula1>=Lists!$B$1:$B$41</formula1>
     </dataValidation>
   </dataValidations>
@@ -6580,7 +6736,7 @@
         <v>11</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
No delivery charge shown; extra cheese on garlic bread and pockets; donair copy
- Delivery charge removed everywhere (home facts, FAQ, order page): it
  differs by area
- Extra cheese tick box on Garlic Bread (sub prices) and Pocket ($4.05)
- Donair poutine: no donair sauce line; donair description names onions
  and tomatoes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TastyPizza-Control.xlsx
+++ b/TastyPizza-Control.xlsx
@@ -664,7 +664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -834,27 +834,12 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>$2.00 | delivery</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>home.facts</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
           <t>Free | parking</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="C16" s="11" t="inlineStr">
+    <row r="15">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>Facts are written as  bold part | the rest  — e.g.  Free | parking</t>
         </is>
@@ -1228,7 +1213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J144"/>
+  <dimension ref="A1:J145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2141,7 +2126,7 @@
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>Spiced beef off the spit, sweet sauce, warm pita. The one we're known for.</t>
+          <t>Spiced beef off the spit with onions, tomatoes and sweet donair sauce on a warm pita. The one we're known for.</t>
         </is>
       </c>
       <c r="E25" s="10" t="n">
@@ -2425,7 +2410,7 @@
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>With donair meat and a line of donair sauce.</t>
+          <t>With donair meat.</t>
         </is>
       </c>
       <c r="E32" s="10" t="n"/>
@@ -3346,45 +3331,33 @@
     <row r="60">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>chicken/Chicken &amp; Chips</t>
+          <t>wraps-pockets/Extra Cheese</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>Chicken</t>
+          <t>Wraps &amp; Pockets</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>Chicken &amp; Chips</t>
+          <t>Extra Cheese</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr"/>
       <c r="E60" s="10" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="F60" s="10" t="n">
-        <v>13.95</v>
-      </c>
-      <c r="G60" s="10" t="n">
-        <v>16.95</v>
-      </c>
+        <v>4.05</v>
+      </c>
+      <c r="F60" s="10" t="n"/>
+      <c r="G60" s="10" t="n"/>
       <c r="H60" s="10" t="n"/>
-      <c r="I60" s="10" t="inlineStr">
-        <is>
-          <t>1 piece / 2 pieces / 3 pieces</t>
-        </is>
-      </c>
-      <c r="J60" s="10" t="inlineStr">
-        <is>
-          <t>fried-chicken</t>
-        </is>
-      </c>
+      <c r="I60" s="10" t="inlineStr"/>
+      <c r="J60" s="10" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>chicken/Extra Piece of Chicken</t>
+          <t>chicken/Chicken &amp; Chips</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
@@ -3394,23 +3367,35 @@
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>Extra Piece of Chicken</t>
+          <t>Chicken &amp; Chips</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr"/>
       <c r="E61" s="10" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="F61" s="10" t="n"/>
-      <c r="G61" s="10" t="n"/>
+        <v>10.95</v>
+      </c>
+      <c r="F61" s="10" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="G61" s="10" t="n">
+        <v>16.95</v>
+      </c>
       <c r="H61" s="10" t="n"/>
-      <c r="I61" s="10" t="inlineStr"/>
-      <c r="J61" s="10" t="inlineStr"/>
+      <c r="I61" s="10" t="inlineStr">
+        <is>
+          <t>1 piece / 2 pieces / 3 pieces</t>
+        </is>
+      </c>
+      <c r="J61" s="10" t="inlineStr">
+        <is>
+          <t>fried-chicken</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>chicken/2 Chicken Legs &amp; Chips</t>
+          <t>chicken/Extra Piece of Chicken</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
@@ -3420,16 +3405,12 @@
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>2 Chicken Legs &amp; Chips</t>
-        </is>
-      </c>
-      <c r="D62" s="10" t="inlineStr">
-        <is>
-          <t>Everyday special.</t>
-        </is>
-      </c>
+          <t>Extra Piece of Chicken</t>
+        </is>
+      </c>
+      <c r="D62" s="10" t="inlineStr"/>
       <c r="E62" s="10" t="n">
-        <v>11.95</v>
+        <v>4.25</v>
       </c>
       <c r="F62" s="10" t="n"/>
       <c r="G62" s="10" t="n"/>
@@ -3440,7 +3421,7 @@
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>chicken/Chicken Family Pack</t>
+          <t>chicken/2 Chicken Legs &amp; Chips</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
@@ -3450,16 +3431,16 @@
       </c>
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>Chicken Family Pack</t>
+          <t>2 Chicken Legs &amp; Chips</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t>10 pieces, 2 large fries, gravy and coleslaw.</t>
+          <t>Everyday special.</t>
         </is>
       </c>
       <c r="E63" s="10" t="n">
-        <v>45.95</v>
+        <v>11.95</v>
       </c>
       <c r="F63" s="10" t="n"/>
       <c r="G63" s="10" t="n"/>
@@ -3470,7 +3451,7 @@
     <row r="64">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>chicken/Chicken Nuggets &amp; Fries</t>
+          <t>chicken/Chicken Family Pack</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
@@ -3480,29 +3461,27 @@
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>Chicken Nuggets &amp; Fries</t>
-        </is>
-      </c>
-      <c r="D64" s="10" t="inlineStr"/>
+          <t>Chicken Family Pack</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="inlineStr">
+        <is>
+          <t>10 pieces, 2 large fries, gravy and coleslaw.</t>
+        </is>
+      </c>
       <c r="E64" s="10" t="n">
-        <v>9.949999999999999</v>
-      </c>
-      <c r="F64" s="10" t="n">
-        <v>17.95</v>
-      </c>
+        <v>45.95</v>
+      </c>
+      <c r="F64" s="10" t="n"/>
       <c r="G64" s="10" t="n"/>
       <c r="H64" s="10" t="n"/>
-      <c r="I64" s="10" t="inlineStr">
-        <is>
-          <t>6 pieces / 12 pieces</t>
-        </is>
-      </c>
+      <c r="I64" s="10" t="inlineStr"/>
       <c r="J64" s="10" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>chicken/Chicken Fingers &amp; Fries</t>
+          <t>chicken/Chicken Nuggets &amp; Fries</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
@@ -3512,63 +3491,65 @@
       </c>
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>Chicken Fingers &amp; Fries</t>
+          <t>Chicken Nuggets &amp; Fries</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr"/>
       <c r="E65" s="10" t="n">
-        <v>16.95</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="F65" s="10" t="n">
-        <v>29.95</v>
+        <v>17.95</v>
       </c>
       <c r="G65" s="10" t="n"/>
       <c r="H65" s="10" t="n"/>
       <c r="I65" s="10" t="inlineStr">
         <is>
-          <t>5 pieces / 10 pieces</t>
-        </is>
-      </c>
-      <c r="J65" s="10" t="inlineStr">
-        <is>
-          <t>chicken-fingers</t>
-        </is>
-      </c>
+          <t>6 pieces / 12 pieces</t>
+        </is>
+      </c>
+      <c r="J65" s="10" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>salads-pasta/Caesar or Garden Salad</t>
+          <t>chicken/Chicken Fingers &amp; Fries</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>Salads &amp; Pasta</t>
+          <t>Chicken</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>Caesar or Garden Salad</t>
+          <t>Chicken Fingers &amp; Fries</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr"/>
       <c r="E66" s="10" t="n">
-        <v>11.45</v>
-      </c>
-      <c r="F66" s="10" t="n"/>
+        <v>16.95</v>
+      </c>
+      <c r="F66" s="10" t="n">
+        <v>29.95</v>
+      </c>
       <c r="G66" s="10" t="n"/>
       <c r="H66" s="10" t="n"/>
-      <c r="I66" s="10" t="inlineStr"/>
+      <c r="I66" s="10" t="inlineStr">
+        <is>
+          <t>5 pieces / 10 pieces</t>
+        </is>
+      </c>
       <c r="J66" s="10" t="inlineStr">
         <is>
-          <t>salad</t>
+          <t>chicken-fingers</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>salads-pasta/Greek Salad</t>
+          <t>salads-pasta/Caesar or Garden Salad</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
@@ -3578,23 +3559,27 @@
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>Greek Salad</t>
+          <t>Caesar or Garden Salad</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr"/>
       <c r="E67" s="10" t="n">
-        <v>12.45</v>
+        <v>11.45</v>
       </c>
       <c r="F67" s="10" t="n"/>
       <c r="G67" s="10" t="n"/>
       <c r="H67" s="10" t="n"/>
       <c r="I67" s="10" t="inlineStr"/>
-      <c r="J67" s="10" t="inlineStr"/>
+      <c r="J67" s="10" t="inlineStr">
+        <is>
+          <t>salad</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>salads-pasta/Lasagna with Garlic Bread</t>
+          <t>salads-pasta/Greek Salad</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
@@ -3604,27 +3589,23 @@
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>Lasagna with Garlic Bread</t>
+          <t>Greek Salad</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr"/>
       <c r="E68" s="10" t="n">
-        <v>13.45</v>
+        <v>12.45</v>
       </c>
       <c r="F68" s="10" t="n"/>
       <c r="G68" s="10" t="n"/>
       <c r="H68" s="10" t="n"/>
       <c r="I68" s="10" t="inlineStr"/>
-      <c r="J68" s="10" t="inlineStr">
-        <is>
-          <t>lasagna</t>
-        </is>
-      </c>
+      <c r="J68" s="10" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>salads-pasta/Ravioli with Garlic Bread</t>
+          <t>salads-pasta/Lasagna with Garlic Bread</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
@@ -3634,7 +3615,7 @@
       </c>
       <c r="C69" s="10" t="inlineStr">
         <is>
-          <t>Ravioli with Garlic Bread</t>
+          <t>Lasagna with Garlic Bread</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr"/>
@@ -3645,46 +3626,42 @@
       <c r="G69" s="10" t="n"/>
       <c r="H69" s="10" t="n"/>
       <c r="I69" s="10" t="inlineStr"/>
-      <c r="J69" s="10" t="inlineStr"/>
+      <c r="J69" s="10" t="inlineStr">
+        <is>
+          <t>lasagna</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="9" t="inlineStr">
         <is>
-          <t>sauces/Donair Sauce</t>
+          <t>salads-pasta/Ravioli with Garlic Bread</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>Sauces</t>
+          <t>Salads &amp; Pasta</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>Donair Sauce</t>
+          <t>Ravioli with Garlic Bread</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr"/>
       <c r="E70" s="10" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F70" s="10" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G70" s="10" t="n">
-        <v>5.25</v>
-      </c>
+        <v>13.45</v>
+      </c>
+      <c r="F70" s="10" t="n"/>
+      <c r="G70" s="10" t="n"/>
       <c r="H70" s="10" t="n"/>
-      <c r="I70" s="10" t="inlineStr">
-        <is>
-          <t>Small / Large / Extra Large</t>
-        </is>
-      </c>
+      <c r="I70" s="10" t="inlineStr"/>
       <c r="J70" s="10" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="9" t="inlineStr">
         <is>
-          <t>sauces/Gravy</t>
+          <t>sauces/Donair Sauce</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
@@ -3694,25 +3671,23 @@
       </c>
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>Gravy</t>
-        </is>
-      </c>
-      <c r="D71" s="10" t="inlineStr">
-        <is>
-          <t>Homemade.</t>
-        </is>
-      </c>
+          <t>Donair Sauce</t>
+        </is>
+      </c>
+      <c r="D71" s="10" t="inlineStr"/>
       <c r="E71" s="10" t="n">
-        <v>1.95</v>
+        <v>2.5</v>
       </c>
       <c r="F71" s="10" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="G71" s="10" t="n"/>
+        <v>3.5</v>
+      </c>
+      <c r="G71" s="10" t="n">
+        <v>5.25</v>
+      </c>
       <c r="H71" s="10" t="n"/>
       <c r="I71" s="10" t="inlineStr">
         <is>
-          <t>Small / Large</t>
+          <t>Small / Large / Extra Large</t>
         </is>
       </c>
       <c r="J71" s="10" t="inlineStr"/>
@@ -3720,33 +3695,43 @@
     <row r="72">
       <c r="A72" s="9" t="inlineStr">
         <is>
-          <t>dips/Cheddar Chipotle Dip</t>
+          <t>sauces/Gravy</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>Dips</t>
+          <t>Sauces</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>Cheddar Chipotle Dip</t>
-        </is>
-      </c>
-      <c r="D72" s="10" t="inlineStr"/>
+          <t>Gravy</t>
+        </is>
+      </c>
+      <c r="D72" s="10" t="inlineStr">
+        <is>
+          <t>Homemade.</t>
+        </is>
+      </c>
       <c r="E72" s="10" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="F72" s="10" t="n"/>
+        <v>1.95</v>
+      </c>
+      <c r="F72" s="10" t="n">
+        <v>3.15</v>
+      </c>
       <c r="G72" s="10" t="n"/>
       <c r="H72" s="10" t="n"/>
-      <c r="I72" s="10" t="inlineStr"/>
+      <c r="I72" s="10" t="inlineStr">
+        <is>
+          <t>Small / Large</t>
+        </is>
+      </c>
       <c r="J72" s="10" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>dips/Creamy Ranch Dip</t>
+          <t>dips/Cheddar Chipotle Dip</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
@@ -3756,7 +3741,7 @@
       </c>
       <c r="C73" s="10" t="inlineStr">
         <is>
-          <t>Creamy Ranch Dip</t>
+          <t>Cheddar Chipotle Dip</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr"/>
@@ -3772,7 +3757,7 @@
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
         <is>
-          <t>dips/Creamy Garlic Dip</t>
+          <t>dips/Creamy Ranch Dip</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
@@ -3782,7 +3767,7 @@
       </c>
       <c r="C74" s="10" t="inlineStr">
         <is>
-          <t>Creamy Garlic Dip</t>
+          <t>Creamy Ranch Dip</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr"/>
@@ -3798,22 +3783,22 @@
     <row r="75">
       <c r="A75" s="9" t="inlineStr">
         <is>
-          <t>beverages/Any 519ml Pop</t>
+          <t>dips/Creamy Garlic Dip</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>Cold Drinks</t>
+          <t>Dips</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
         <is>
-          <t>Any 519ml Pop</t>
+          <t>Creamy Garlic Dip</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr"/>
       <c r="E75" s="10" t="n">
-        <v>2.59</v>
+        <v>1.75</v>
       </c>
       <c r="F75" s="10" t="n"/>
       <c r="G75" s="10" t="n"/>
@@ -3824,7 +3809,7 @@
     <row r="76">
       <c r="A76" s="9" t="inlineStr">
         <is>
-          <t>beverages/Any Juice, Gatorade, G2 or Energy Drink</t>
+          <t>beverages/Any 519ml Pop</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
@@ -3834,12 +3819,12 @@
       </c>
       <c r="C76" s="10" t="inlineStr">
         <is>
-          <t>Any Juice, Gatorade, G2 or Energy Drink</t>
+          <t>Any 519ml Pop</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr"/>
       <c r="E76" s="10" t="n">
-        <v>3.39</v>
+        <v>2.59</v>
       </c>
       <c r="F76" s="10" t="n"/>
       <c r="G76" s="10" t="n"/>
@@ -3850,7 +3835,7 @@
     <row r="77">
       <c r="A77" s="9" t="inlineStr">
         <is>
-          <t>beverages/Chocolate Milk</t>
+          <t>beverages/Any Juice, Gatorade, G2 or Energy Drink</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
@@ -3860,12 +3845,12 @@
       </c>
       <c r="C77" s="10" t="inlineStr">
         <is>
-          <t>Chocolate Milk</t>
+          <t>Any Juice, Gatorade, G2 or Energy Drink</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr"/>
       <c r="E77" s="10" t="n">
-        <v>2.79</v>
+        <v>3.39</v>
       </c>
       <c r="F77" s="10" t="n"/>
       <c r="G77" s="10" t="n"/>
@@ -3876,7 +3861,7 @@
     <row r="78">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>beverages/Any 355ml Pop</t>
+          <t>beverages/Chocolate Milk</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
@@ -3886,12 +3871,12 @@
       </c>
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>Any 355ml Pop</t>
+          <t>Chocolate Milk</t>
         </is>
       </c>
       <c r="D78" s="10" t="inlineStr"/>
       <c r="E78" s="10" t="n">
-        <v>1.59</v>
+        <v>2.79</v>
       </c>
       <c r="F78" s="10" t="n"/>
       <c r="G78" s="10" t="n"/>
@@ -3902,7 +3887,7 @@
     <row r="79">
       <c r="A79" s="9" t="inlineStr">
         <is>
-          <t>beverages/Any 2L Pop</t>
+          <t>beverages/Any 355ml Pop</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
@@ -3912,12 +3897,12 @@
       </c>
       <c r="C79" s="10" t="inlineStr">
         <is>
-          <t>Any 2L Pop</t>
+          <t>Any 355ml Pop</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr"/>
       <c r="E79" s="10" t="n">
-        <v>4.19</v>
+        <v>1.59</v>
       </c>
       <c r="F79" s="10" t="n"/>
       <c r="G79" s="10" t="n"/>
@@ -3928,7 +3913,7 @@
     <row r="80">
       <c r="A80" s="9" t="inlineStr">
         <is>
-          <t>beverages/Aquafina Water 591ml</t>
+          <t>beverages/Any 2L Pop</t>
         </is>
       </c>
       <c r="B80" s="10" t="inlineStr">
@@ -3938,12 +3923,12 @@
       </c>
       <c r="C80" s="10" t="inlineStr">
         <is>
-          <t>Aquafina Water 591ml</t>
+          <t>Any 2L Pop</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr"/>
       <c r="E80" s="10" t="n">
-        <v>1.69</v>
+        <v>4.19</v>
       </c>
       <c r="F80" s="10" t="n"/>
       <c r="G80" s="10" t="n"/>
@@ -3954,49 +3939,33 @@
     <row r="81">
       <c r="A81" s="9" t="inlineStr">
         <is>
-          <t>fish/Fish &amp; Chips</t>
+          <t>beverages/Aquafina Water 591ml</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>Fish &amp; Chips</t>
+          <t>Cold Drinks</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
         <is>
-          <t>Fish &amp; Chips</t>
-        </is>
-      </c>
-      <c r="D81" s="10" t="inlineStr">
-        <is>
-          <t>Fresh haddock and fries.</t>
-        </is>
-      </c>
+          <t>Aquafina Water 591ml</t>
+        </is>
+      </c>
+      <c r="D81" s="10" t="inlineStr"/>
       <c r="E81" s="10" t="n">
-        <v>11.95</v>
-      </c>
-      <c r="F81" s="10" t="n">
-        <v>15.95</v>
-      </c>
-      <c r="G81" s="10" t="n">
-        <v>17.95</v>
-      </c>
+        <v>1.69</v>
+      </c>
+      <c r="F81" s="10" t="n"/>
+      <c r="G81" s="10" t="n"/>
       <c r="H81" s="10" t="n"/>
-      <c r="I81" s="10" t="inlineStr">
-        <is>
-          <t>1 piece / 2 pieces / 3 pieces</t>
-        </is>
-      </c>
-      <c r="J81" s="10" t="inlineStr">
-        <is>
-          <t>fish-and-chips</t>
-        </is>
-      </c>
+      <c r="I81" s="10" t="inlineStr"/>
+      <c r="J81" s="10" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="9" t="inlineStr">
         <is>
-          <t>fish/Extra Piece of Fish</t>
+          <t>fish/Fish &amp; Chips</t>
         </is>
       </c>
       <c r="B82" s="10" t="inlineStr">
@@ -4006,23 +3975,39 @@
       </c>
       <c r="C82" s="10" t="inlineStr">
         <is>
-          <t>Extra Piece of Fish</t>
-        </is>
-      </c>
-      <c r="D82" s="10" t="inlineStr"/>
+          <t>Fish &amp; Chips</t>
+        </is>
+      </c>
+      <c r="D82" s="10" t="inlineStr">
+        <is>
+          <t>Fresh haddock and fries.</t>
+        </is>
+      </c>
       <c r="E82" s="10" t="n">
-        <v>4.95</v>
-      </c>
-      <c r="F82" s="10" t="n"/>
-      <c r="G82" s="10" t="n"/>
+        <v>11.95</v>
+      </c>
+      <c r="F82" s="10" t="n">
+        <v>15.95</v>
+      </c>
+      <c r="G82" s="10" t="n">
+        <v>17.95</v>
+      </c>
       <c r="H82" s="10" t="n"/>
-      <c r="I82" s="10" t="inlineStr"/>
-      <c r="J82" s="10" t="inlineStr"/>
+      <c r="I82" s="10" t="inlineStr">
+        <is>
+          <t>1 piece / 2 pieces / 3 pieces</t>
+        </is>
+      </c>
+      <c r="J82" s="10" t="inlineStr">
+        <is>
+          <t>fish-and-chips</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="9" t="inlineStr">
         <is>
-          <t>fish/Fish Family Pack</t>
+          <t>fish/Extra Piece of Fish</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
@@ -4032,16 +4017,12 @@
       </c>
       <c r="C83" s="10" t="inlineStr">
         <is>
-          <t>Fish Family Pack</t>
-        </is>
-      </c>
-      <c r="D83" s="10" t="inlineStr">
-        <is>
-          <t>10 pieces of fish, 2 large fries, large gravy, coleslaw and tartar sauce.</t>
-        </is>
-      </c>
+          <t>Extra Piece of Fish</t>
+        </is>
+      </c>
+      <c r="D83" s="10" t="inlineStr"/>
       <c r="E83" s="10" t="n">
-        <v>46.95</v>
+        <v>4.95</v>
       </c>
       <c r="F83" s="10" t="n"/>
       <c r="G83" s="10" t="n"/>
@@ -4052,41 +4033,37 @@
     <row r="84">
       <c r="A84" s="9" t="inlineStr">
         <is>
-          <t>seafood/Scallops &amp; Chips</t>
+          <t>fish/Fish Family Pack</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t>More Seafood</t>
+          <t>Fish &amp; Chips</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
         <is>
-          <t>Scallops &amp; Chips</t>
+          <t>Fish Family Pack</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t>10 scallops.</t>
+          <t>10 pieces of fish, 2 large fries, large gravy, coleslaw and tartar sauce.</t>
         </is>
       </c>
       <c r="E84" s="10" t="n">
-        <v>14.95</v>
+        <v>46.95</v>
       </c>
       <c r="F84" s="10" t="n"/>
       <c r="G84" s="10" t="n"/>
       <c r="H84" s="10" t="n"/>
       <c r="I84" s="10" t="inlineStr"/>
-      <c r="J84" s="10" t="inlineStr">
-        <is>
-          <t>scallops</t>
-        </is>
-      </c>
+      <c r="J84" s="10" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="9" t="inlineStr">
         <is>
-          <t>seafood/Clams &amp; Chips</t>
+          <t>seafood/Scallops &amp; Chips</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
@@ -4096,12 +4073,12 @@
       </c>
       <c r="C85" s="10" t="inlineStr">
         <is>
-          <t>Clams &amp; Chips</t>
+          <t>Scallops &amp; Chips</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t>Two cups of clams.</t>
+          <t>10 scallops.</t>
         </is>
       </c>
       <c r="E85" s="10" t="n">
@@ -4111,12 +4088,16 @@
       <c r="G85" s="10" t="n"/>
       <c r="H85" s="10" t="n"/>
       <c r="I85" s="10" t="inlineStr"/>
-      <c r="J85" s="10" t="inlineStr"/>
+      <c r="J85" s="10" t="inlineStr">
+        <is>
+          <t>scallops</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="9" t="inlineStr">
         <is>
-          <t>seafood/Shrimp &amp; Chips</t>
+          <t>seafood/Clams &amp; Chips</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
@@ -4126,12 +4107,12 @@
       </c>
       <c r="C86" s="10" t="inlineStr">
         <is>
-          <t>Shrimp &amp; Chips</t>
+          <t>Clams &amp; Chips</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
         <is>
-          <t>12 shrimp.</t>
+          <t>Two cups of clams.</t>
         </is>
       </c>
       <c r="E86" s="10" t="n">
@@ -4141,16 +4122,12 @@
       <c r="G86" s="10" t="n"/>
       <c r="H86" s="10" t="n"/>
       <c r="I86" s="10" t="inlineStr"/>
-      <c r="J86" s="10" t="inlineStr">
-        <is>
-          <t>shrimp</t>
-        </is>
-      </c>
+      <c r="J86" s="10" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="9" t="inlineStr">
         <is>
-          <t>seafood/Seafood Platter</t>
+          <t>seafood/Shrimp &amp; Chips</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
@@ -4160,27 +4137,31 @@
       </c>
       <c r="C87" s="10" t="inlineStr">
         <is>
-          <t>Seafood Platter</t>
+          <t>Shrimp &amp; Chips</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t>A piece of fish, fries, 5 scallops, 5 shrimp and clams.</t>
+          <t>12 shrimp.</t>
         </is>
       </c>
       <c r="E87" s="10" t="n">
-        <v>23.95</v>
+        <v>14.95</v>
       </c>
       <c r="F87" s="10" t="n"/>
       <c r="G87" s="10" t="n"/>
       <c r="H87" s="10" t="n"/>
       <c r="I87" s="10" t="inlineStr"/>
-      <c r="J87" s="10" t="inlineStr"/>
+      <c r="J87" s="10" t="inlineStr">
+        <is>
+          <t>shrimp</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="9" t="inlineStr">
         <is>
-          <t>seafood/Extra Coleslaw</t>
+          <t>seafood/Seafood Platter</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
@@ -4190,47 +4171,45 @@
       </c>
       <c r="C88" s="10" t="inlineStr">
         <is>
-          <t>Extra Coleslaw</t>
-        </is>
-      </c>
-      <c r="D88" s="10" t="inlineStr"/>
+          <t>Seafood Platter</t>
+        </is>
+      </c>
+      <c r="D88" s="10" t="inlineStr">
+        <is>
+          <t>A piece of fish, fries, 5 scallops, 5 shrimp and clams.</t>
+        </is>
+      </c>
       <c r="E88" s="10" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="F88" s="10" t="n">
-        <v>3.45</v>
-      </c>
+        <v>23.95</v>
+      </c>
+      <c r="F88" s="10" t="n"/>
       <c r="G88" s="10" t="n"/>
       <c r="H88" s="10" t="n"/>
-      <c r="I88" s="10" t="inlineStr">
-        <is>
-          <t>Small / Large</t>
-        </is>
-      </c>
+      <c r="I88" s="10" t="inlineStr"/>
       <c r="J88" s="10" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="9" t="inlineStr">
         <is>
-          <t>subs/Cold Cut</t>
+          <t>seafood/Extra Coleslaw</t>
         </is>
       </c>
       <c r="B89" s="10" t="inlineStr">
         <is>
-          <t>Subs</t>
+          <t>More Seafood</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
         <is>
-          <t>Cold Cut</t>
+          <t>Extra Coleslaw</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr"/>
       <c r="E89" s="10" t="n">
-        <v>10.95</v>
+        <v>2.25</v>
       </c>
       <c r="F89" s="10" t="n">
-        <v>13.25</v>
+        <v>3.45</v>
       </c>
       <c r="G89" s="10" t="n"/>
       <c r="H89" s="10" t="n"/>
@@ -4239,16 +4218,12 @@
           <t>Small / Large</t>
         </is>
       </c>
-      <c r="J89" s="10" t="inlineStr">
-        <is>
-          <t>cold-cut-sub</t>
-        </is>
-      </c>
+      <c r="J89" s="10" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="9" t="inlineStr">
         <is>
-          <t>subs/Salami &amp; Ham</t>
+          <t>subs/Cold Cut</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
@@ -4258,7 +4233,7 @@
       </c>
       <c r="C90" s="10" t="inlineStr">
         <is>
-          <t>Salami &amp; Ham</t>
+          <t>Cold Cut</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr"/>
@@ -4275,12 +4250,16 @@
           <t>Small / Large</t>
         </is>
       </c>
-      <c r="J90" s="10" t="inlineStr"/>
+      <c r="J90" s="10" t="inlineStr">
+        <is>
+          <t>cold-cut-sub</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="9" t="inlineStr">
         <is>
-          <t>subs/Pizza Sub</t>
+          <t>subs/Salami &amp; Ham</t>
         </is>
       </c>
       <c r="B91" s="10" t="inlineStr">
@@ -4290,7 +4269,7 @@
       </c>
       <c r="C91" s="10" t="inlineStr">
         <is>
-          <t>Pizza Sub</t>
+          <t>Salami &amp; Ham</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr"/>
@@ -4312,7 +4291,7 @@
     <row r="92">
       <c r="A92" s="9" t="inlineStr">
         <is>
-          <t>subs/Vegetarian</t>
+          <t>subs/Pizza Sub</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
@@ -4322,7 +4301,7 @@
       </c>
       <c r="C92" s="10" t="inlineStr">
         <is>
-          <t>Vegetarian</t>
+          <t>Pizza Sub</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr"/>
@@ -4344,7 +4323,7 @@
     <row r="93">
       <c r="A93" s="9" t="inlineStr">
         <is>
-          <t>subs/Real Turkey</t>
+          <t>subs/Vegetarian</t>
         </is>
       </c>
       <c r="B93" s="10" t="inlineStr">
@@ -4354,12 +4333,12 @@
       </c>
       <c r="C93" s="10" t="inlineStr">
         <is>
-          <t>Real Turkey</t>
+          <t>Vegetarian</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr"/>
       <c r="E93" s="10" t="n">
-        <v>11.45</v>
+        <v>10.95</v>
       </c>
       <c r="F93" s="10" t="n">
         <v>13.25</v>
@@ -4376,7 +4355,7 @@
     <row r="94">
       <c r="A94" s="9" t="inlineStr">
         <is>
-          <t>subs/Bubba</t>
+          <t>subs/Real Turkey</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
@@ -4386,19 +4365,15 @@
       </c>
       <c r="C94" s="10" t="inlineStr">
         <is>
-          <t>Bubba</t>
-        </is>
-      </c>
-      <c r="D94" s="10" t="inlineStr">
-        <is>
-          <t>The one people ask for by name.</t>
-        </is>
-      </c>
+          <t>Real Turkey</t>
+        </is>
+      </c>
+      <c r="D94" s="10" t="inlineStr"/>
       <c r="E94" s="10" t="n">
-        <v>11.95</v>
+        <v>11.45</v>
       </c>
       <c r="F94" s="10" t="n">
-        <v>14.25</v>
+        <v>13.25</v>
       </c>
       <c r="G94" s="10" t="n"/>
       <c r="H94" s="10" t="n"/>
@@ -4412,7 +4387,7 @@
     <row r="95">
       <c r="A95" s="9" t="inlineStr">
         <is>
-          <t>subs/Club</t>
+          <t>subs/Bubba</t>
         </is>
       </c>
       <c r="B95" s="10" t="inlineStr">
@@ -4422,10 +4397,14 @@
       </c>
       <c r="C95" s="10" t="inlineStr">
         <is>
-          <t>Club</t>
-        </is>
-      </c>
-      <c r="D95" s="10" t="inlineStr"/>
+          <t>Bubba</t>
+        </is>
+      </c>
+      <c r="D95" s="10" t="inlineStr">
+        <is>
+          <t>The one people ask for by name.</t>
+        </is>
+      </c>
       <c r="E95" s="10" t="n">
         <v>11.95</v>
       </c>
@@ -4444,7 +4423,7 @@
     <row r="96">
       <c r="A96" s="9" t="inlineStr">
         <is>
-          <t>subs/Steak</t>
+          <t>subs/Club</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
@@ -4454,7 +4433,7 @@
       </c>
       <c r="C96" s="10" t="inlineStr">
         <is>
-          <t>Steak</t>
+          <t>Club</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr"/>
@@ -4462,7 +4441,7 @@
         <v>11.95</v>
       </c>
       <c r="F96" s="10" t="n">
-        <v>14.95</v>
+        <v>14.25</v>
       </c>
       <c r="G96" s="10" t="n"/>
       <c r="H96" s="10" t="n"/>
@@ -4471,16 +4450,12 @@
           <t>Small / Large</t>
         </is>
       </c>
-      <c r="J96" s="10" t="inlineStr">
-        <is>
-          <t>steak-sub</t>
-        </is>
-      </c>
+      <c r="J96" s="10" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="9" t="inlineStr">
         <is>
-          <t>subs/Donair Sub</t>
+          <t>subs/Steak</t>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
@@ -4490,7 +4465,7 @@
       </c>
       <c r="C97" s="10" t="inlineStr">
         <is>
-          <t>Donair Sub</t>
+          <t>Steak</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr"/>
@@ -4507,12 +4482,16 @@
           <t>Small / Large</t>
         </is>
       </c>
-      <c r="J97" s="10" t="inlineStr"/>
+      <c r="J97" s="10" t="inlineStr">
+        <is>
+          <t>steak-sub</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="9" t="inlineStr">
         <is>
-          <t>subs/Super Sub</t>
+          <t>subs/Donair Sub</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
@@ -4522,15 +4501,15 @@
       </c>
       <c r="C98" s="10" t="inlineStr">
         <is>
-          <t>Super Sub</t>
+          <t>Donair Sub</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr"/>
       <c r="E98" s="10" t="n">
-        <v>12.45</v>
+        <v>11.95</v>
       </c>
       <c r="F98" s="10" t="n">
-        <v>16.25</v>
+        <v>14.95</v>
       </c>
       <c r="G98" s="10" t="n"/>
       <c r="H98" s="10" t="n"/>
@@ -4544,7 +4523,7 @@
     <row r="99">
       <c r="A99" s="9" t="inlineStr">
         <is>
-          <t>subs/Garlic Bread</t>
+          <t>subs/Super Sub</t>
         </is>
       </c>
       <c r="B99" s="10" t="inlineStr">
@@ -4554,15 +4533,15 @@
       </c>
       <c r="C99" s="10" t="inlineStr">
         <is>
-          <t>Garlic Bread</t>
+          <t>Super Sub</t>
         </is>
       </c>
       <c r="D99" s="10" t="inlineStr"/>
       <c r="E99" s="10" t="n">
-        <v>6.25</v>
+        <v>12.45</v>
       </c>
       <c r="F99" s="10" t="n">
-        <v>7.45</v>
+        <v>16.25</v>
       </c>
       <c r="G99" s="10" t="n"/>
       <c r="H99" s="10" t="n"/>
@@ -4576,7 +4555,7 @@
     <row r="100">
       <c r="A100" s="9" t="inlineStr">
         <is>
-          <t>subs/Extra Cheese</t>
+          <t>subs/Garlic Bread</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
@@ -4586,15 +4565,15 @@
       </c>
       <c r="C100" s="10" t="inlineStr">
         <is>
-          <t>Extra Cheese</t>
+          <t>Garlic Bread</t>
         </is>
       </c>
       <c r="D100" s="10" t="inlineStr"/>
       <c r="E100" s="10" t="n">
-        <v>2.75</v>
+        <v>6.25</v>
       </c>
       <c r="F100" s="10" t="n">
-        <v>3.95</v>
+        <v>7.45</v>
       </c>
       <c r="G100" s="10" t="n"/>
       <c r="H100" s="10" t="n"/>
@@ -4608,7 +4587,7 @@
     <row r="101">
       <c r="A101" s="9" t="inlineStr">
         <is>
-          <t>subs/Extra Meat</t>
+          <t>subs/Extra Cheese</t>
         </is>
       </c>
       <c r="B101" s="10" t="inlineStr">
@@ -4618,15 +4597,15 @@
       </c>
       <c r="C101" s="10" t="inlineStr">
         <is>
-          <t>Extra Meat</t>
+          <t>Extra Cheese</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr"/>
       <c r="E101" s="10" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="F101" s="10" t="n">
         <v>3.95</v>
-      </c>
-      <c r="F101" s="10" t="n">
-        <v>4.75</v>
       </c>
       <c r="G101" s="10" t="n"/>
       <c r="H101" s="10" t="n"/>
@@ -4640,33 +4619,31 @@
     <row r="102">
       <c r="A102" s="9" t="inlineStr">
         <is>
-          <t>burritos/Beans &amp; Veggie</t>
+          <t>subs/Extra Meat</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t>Burritos</t>
+          <t>Subs</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
         <is>
-          <t>Beans &amp; Veggie</t>
+          <t>Extra Meat</t>
         </is>
       </c>
       <c r="D102" s="10" t="inlineStr"/>
       <c r="E102" s="10" t="n">
-        <v>7.99</v>
+        <v>3.95</v>
       </c>
       <c r="F102" s="10" t="n">
-        <v>8.99</v>
-      </c>
-      <c r="G102" s="10" t="n">
-        <v>10.99</v>
-      </c>
+        <v>4.75</v>
+      </c>
+      <c r="G102" s="10" t="n"/>
       <c r="H102" s="10" t="n"/>
       <c r="I102" s="10" t="inlineStr">
         <is>
-          <t>Small / Medium / Large</t>
+          <t>Small / Large</t>
         </is>
       </c>
       <c r="J102" s="10" t="inlineStr"/>
@@ -4674,7 +4651,7 @@
     <row r="103">
       <c r="A103" s="9" t="inlineStr">
         <is>
-          <t>burritos/Spicy Chicken</t>
+          <t>burritos/Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="B103" s="10" t="inlineStr">
@@ -4684,18 +4661,18 @@
       </c>
       <c r="C103" s="10" t="inlineStr">
         <is>
-          <t>Spicy Chicken</t>
+          <t>Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr"/>
       <c r="E103" s="10" t="n">
-        <v>9.99</v>
+        <v>7.99</v>
       </c>
       <c r="F103" s="10" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="G103" s="10" t="n">
         <v>10.99</v>
-      </c>
-      <c r="G103" s="10" t="n">
-        <v>12.99</v>
       </c>
       <c r="H103" s="10" t="n"/>
       <c r="I103" s="10" t="inlineStr">
@@ -4703,16 +4680,12 @@
           <t>Small / Medium / Large</t>
         </is>
       </c>
-      <c r="J103" s="10" t="inlineStr">
-        <is>
-          <t>burrito</t>
-        </is>
-      </c>
+      <c r="J103" s="10" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="9" t="inlineStr">
         <is>
-          <t>burritos/Ground Beef</t>
+          <t>burritos/Spicy Chicken</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
@@ -4722,7 +4695,7 @@
       </c>
       <c r="C104" s="10" t="inlineStr">
         <is>
-          <t>Ground Beef</t>
+          <t>Spicy Chicken</t>
         </is>
       </c>
       <c r="D104" s="10" t="inlineStr"/>
@@ -4741,12 +4714,16 @@
           <t>Small / Medium / Large</t>
         </is>
       </c>
-      <c r="J104" s="10" t="inlineStr"/>
+      <c r="J104" s="10" t="inlineStr">
+        <is>
+          <t>burrito</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="9" t="inlineStr">
         <is>
-          <t>burritos/Zesty Grilled Chicken</t>
+          <t>burritos/Ground Beef</t>
         </is>
       </c>
       <c r="B105" s="10" t="inlineStr">
@@ -4756,7 +4733,7 @@
       </c>
       <c r="C105" s="10" t="inlineStr">
         <is>
-          <t>Zesty Grilled Chicken</t>
+          <t>Ground Beef</t>
         </is>
       </c>
       <c r="D105" s="10" t="inlineStr"/>
@@ -4780,7 +4757,7 @@
     <row r="106">
       <c r="A106" s="9" t="inlineStr">
         <is>
-          <t>burritos/Fish</t>
+          <t>burritos/Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
@@ -4790,7 +4767,7 @@
       </c>
       <c r="C106" s="10" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="D106" s="10" t="inlineStr"/>
@@ -4814,7 +4791,7 @@
     <row r="107">
       <c r="A107" s="9" t="inlineStr">
         <is>
-          <t>burritos/Shawarma Chicken</t>
+          <t>burritos/Fish</t>
         </is>
       </c>
       <c r="B107" s="10" t="inlineStr">
@@ -4824,18 +4801,18 @@
       </c>
       <c r="C107" s="10" t="inlineStr">
         <is>
-          <t>Shawarma Chicken</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D107" s="10" t="inlineStr"/>
       <c r="E107" s="10" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="F107" s="10" t="n">
         <v>10.99</v>
       </c>
-      <c r="F107" s="10" t="n">
-        <v>11.99</v>
-      </c>
       <c r="G107" s="10" t="n">
-        <v>13.99</v>
+        <v>12.99</v>
       </c>
       <c r="H107" s="10" t="n"/>
       <c r="I107" s="10" t="inlineStr">
@@ -4848,7 +4825,7 @@
     <row r="108">
       <c r="A108" s="9" t="inlineStr">
         <is>
-          <t>burritos/Tequila-Lime Glazed Chicken</t>
+          <t>burritos/Shawarma Chicken</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
@@ -4858,7 +4835,7 @@
       </c>
       <c r="C108" s="10" t="inlineStr">
         <is>
-          <t>Tequila-Lime Glazed Chicken</t>
+          <t>Shawarma Chicken</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr"/>
@@ -4882,7 +4859,7 @@
     <row r="109">
       <c r="A109" s="9" t="inlineStr">
         <is>
-          <t>burritos/Steak</t>
+          <t>burritos/Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
@@ -4892,7 +4869,7 @@
       </c>
       <c r="C109" s="10" t="inlineStr">
         <is>
-          <t>Steak</t>
+          <t>Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr"/>
@@ -4916,43 +4893,41 @@
     <row r="110">
       <c r="A110" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Beans &amp; Veggie</t>
+          <t>burritos/Steak</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t>Rice Bowls</t>
+          <t>Burritos</t>
         </is>
       </c>
       <c r="C110" s="10" t="inlineStr">
         <is>
-          <t>Beans &amp; Veggie</t>
+          <t>Steak</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr"/>
       <c r="E110" s="10" t="n">
-        <v>10.49</v>
+        <v>10.99</v>
       </c>
       <c r="F110" s="10" t="n">
-        <v>12.49</v>
-      </c>
-      <c r="G110" s="10" t="n"/>
+        <v>11.99</v>
+      </c>
+      <c r="G110" s="10" t="n">
+        <v>13.99</v>
+      </c>
       <c r="H110" s="10" t="n"/>
       <c r="I110" s="10" t="inlineStr">
         <is>
-          <t>Small / Large</t>
-        </is>
-      </c>
-      <c r="J110" s="10" t="inlineStr">
-        <is>
-          <t>rice-bowl</t>
-        </is>
-      </c>
+          <t>Small / Medium / Large</t>
+        </is>
+      </c>
+      <c r="J110" s="10" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Spicy Chicken</t>
+          <t>rice-bowls/Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="B111" s="10" t="inlineStr">
@@ -4962,15 +4937,15 @@
       </c>
       <c r="C111" s="10" t="inlineStr">
         <is>
-          <t>Spicy Chicken</t>
+          <t>Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr"/>
       <c r="E111" s="10" t="n">
-        <v>11.49</v>
+        <v>10.49</v>
       </c>
       <c r="F111" s="10" t="n">
-        <v>13.49</v>
+        <v>12.49</v>
       </c>
       <c r="G111" s="10" t="n"/>
       <c r="H111" s="10" t="n"/>
@@ -4979,12 +4954,16 @@
           <t>Small / Large</t>
         </is>
       </c>
-      <c r="J111" s="10" t="inlineStr"/>
+      <c r="J111" s="10" t="inlineStr">
+        <is>
+          <t>rice-bowl</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Ground Beef</t>
+          <t>rice-bowls/Spicy Chicken</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
@@ -4994,7 +4973,7 @@
       </c>
       <c r="C112" s="10" t="inlineStr">
         <is>
-          <t>Ground Beef</t>
+          <t>Spicy Chicken</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr"/>
@@ -5016,7 +4995,7 @@
     <row r="113">
       <c r="A113" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Zesty Grilled Chicken</t>
+          <t>rice-bowls/Ground Beef</t>
         </is>
       </c>
       <c r="B113" s="10" t="inlineStr">
@@ -5026,7 +5005,7 @@
       </c>
       <c r="C113" s="10" t="inlineStr">
         <is>
-          <t>Zesty Grilled Chicken</t>
+          <t>Ground Beef</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr"/>
@@ -5048,7 +5027,7 @@
     <row r="114">
       <c r="A114" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Fish</t>
+          <t>rice-bowls/Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
@@ -5058,7 +5037,7 @@
       </c>
       <c r="C114" s="10" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr"/>
@@ -5080,7 +5059,7 @@
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Shawarma Chicken</t>
+          <t>rice-bowls/Fish</t>
         </is>
       </c>
       <c r="B115" s="10" t="inlineStr">
@@ -5090,15 +5069,15 @@
       </c>
       <c r="C115" s="10" t="inlineStr">
         <is>
-          <t>Shawarma Chicken</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D115" s="10" t="inlineStr"/>
       <c r="E115" s="10" t="n">
-        <v>12.49</v>
+        <v>11.49</v>
       </c>
       <c r="F115" s="10" t="n">
-        <v>14.49</v>
+        <v>13.49</v>
       </c>
       <c r="G115" s="10" t="n"/>
       <c r="H115" s="10" t="n"/>
@@ -5112,7 +5091,7 @@
     <row r="116">
       <c r="A116" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Tequila-Lime Glazed Chicken</t>
+          <t>rice-bowls/Shawarma Chicken</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
@@ -5122,7 +5101,7 @@
       </c>
       <c r="C116" s="10" t="inlineStr">
         <is>
-          <t>Tequila-Lime Glazed Chicken</t>
+          <t>Shawarma Chicken</t>
         </is>
       </c>
       <c r="D116" s="10" t="inlineStr"/>
@@ -5144,7 +5123,7 @@
     <row r="117">
       <c r="A117" s="9" t="inlineStr">
         <is>
-          <t>rice-bowls/Steak</t>
+          <t>rice-bowls/Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="B117" s="10" t="inlineStr">
@@ -5154,7 +5133,7 @@
       </c>
       <c r="C117" s="10" t="inlineStr">
         <is>
-          <t>Steak</t>
+          <t>Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="D117" s="10" t="inlineStr"/>
@@ -5176,37 +5155,39 @@
     <row r="118">
       <c r="A118" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Beans &amp; Veggie</t>
+          <t>rice-bowls/Steak</t>
         </is>
       </c>
       <c r="B118" s="10" t="inlineStr">
         <is>
-          <t>Quesadillas</t>
+          <t>Rice Bowls</t>
         </is>
       </c>
       <c r="C118" s="10" t="inlineStr">
         <is>
-          <t>Beans &amp; Veggie</t>
+          <t>Steak</t>
         </is>
       </c>
       <c r="D118" s="10" t="inlineStr"/>
       <c r="E118" s="10" t="n">
-        <v>10.49</v>
-      </c>
-      <c r="F118" s="10" t="n"/>
+        <v>12.49</v>
+      </c>
+      <c r="F118" s="10" t="n">
+        <v>14.49</v>
+      </c>
       <c r="G118" s="10" t="n"/>
       <c r="H118" s="10" t="n"/>
-      <c r="I118" s="10" t="inlineStr"/>
-      <c r="J118" s="10" t="inlineStr">
-        <is>
-          <t>quesadilla</t>
-        </is>
-      </c>
+      <c r="I118" s="10" t="inlineStr">
+        <is>
+          <t>Small / Large</t>
+        </is>
+      </c>
+      <c r="J118" s="10" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Spicy Chicken</t>
+          <t>quesadillas/Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="B119" s="10" t="inlineStr">
@@ -5216,23 +5197,27 @@
       </c>
       <c r="C119" s="10" t="inlineStr">
         <is>
-          <t>Spicy Chicken</t>
+          <t>Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="D119" s="10" t="inlineStr"/>
       <c r="E119" s="10" t="n">
-        <v>11.49</v>
+        <v>10.49</v>
       </c>
       <c r="F119" s="10" t="n"/>
       <c r="G119" s="10" t="n"/>
       <c r="H119" s="10" t="n"/>
       <c r="I119" s="10" t="inlineStr"/>
-      <c r="J119" s="10" t="inlineStr"/>
+      <c r="J119" s="10" t="inlineStr">
+        <is>
+          <t>quesadilla</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Ground Beef</t>
+          <t>quesadillas/Spicy Chicken</t>
         </is>
       </c>
       <c r="B120" s="10" t="inlineStr">
@@ -5242,7 +5227,7 @@
       </c>
       <c r="C120" s="10" t="inlineStr">
         <is>
-          <t>Ground Beef</t>
+          <t>Spicy Chicken</t>
         </is>
       </c>
       <c r="D120" s="10" t="inlineStr"/>
@@ -5258,7 +5243,7 @@
     <row r="121">
       <c r="A121" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Zesty Grilled Chicken</t>
+          <t>quesadillas/Ground Beef</t>
         </is>
       </c>
       <c r="B121" s="10" t="inlineStr">
@@ -5268,7 +5253,7 @@
       </c>
       <c r="C121" s="10" t="inlineStr">
         <is>
-          <t>Zesty Grilled Chicken</t>
+          <t>Ground Beef</t>
         </is>
       </c>
       <c r="D121" s="10" t="inlineStr"/>
@@ -5284,7 +5269,7 @@
     <row r="122">
       <c r="A122" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Fish</t>
+          <t>quesadillas/Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="B122" s="10" t="inlineStr">
@@ -5294,7 +5279,7 @@
       </c>
       <c r="C122" s="10" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr"/>
@@ -5310,7 +5295,7 @@
     <row r="123">
       <c r="A123" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Shawarma Chicken</t>
+          <t>quesadillas/Fish</t>
         </is>
       </c>
       <c r="B123" s="10" t="inlineStr">
@@ -5320,12 +5305,12 @@
       </c>
       <c r="C123" s="10" t="inlineStr">
         <is>
-          <t>Shawarma Chicken</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D123" s="10" t="inlineStr"/>
       <c r="E123" s="10" t="n">
-        <v>12.49</v>
+        <v>11.49</v>
       </c>
       <c r="F123" s="10" t="n"/>
       <c r="G123" s="10" t="n"/>
@@ -5336,7 +5321,7 @@
     <row r="124">
       <c r="A124" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Tequila-Lime Glazed Chicken</t>
+          <t>quesadillas/Shawarma Chicken</t>
         </is>
       </c>
       <c r="B124" s="10" t="inlineStr">
@@ -5346,7 +5331,7 @@
       </c>
       <c r="C124" s="10" t="inlineStr">
         <is>
-          <t>Tequila-Lime Glazed Chicken</t>
+          <t>Shawarma Chicken</t>
         </is>
       </c>
       <c r="D124" s="10" t="inlineStr"/>
@@ -5362,7 +5347,7 @@
     <row r="125">
       <c r="A125" s="9" t="inlineStr">
         <is>
-          <t>quesadillas/Steak</t>
+          <t>quesadillas/Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="B125" s="10" t="inlineStr">
@@ -5372,7 +5357,7 @@
       </c>
       <c r="C125" s="10" t="inlineStr">
         <is>
-          <t>Steak</t>
+          <t>Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr"/>
@@ -5388,37 +5373,33 @@
     <row r="126">
       <c r="A126" s="9" t="inlineStr">
         <is>
-          <t>tacos/Beans &amp; Veggie</t>
+          <t>quesadillas/Steak</t>
         </is>
       </c>
       <c r="B126" s="10" t="inlineStr">
         <is>
-          <t>Tacos</t>
+          <t>Quesadillas</t>
         </is>
       </c>
       <c r="C126" s="10" t="inlineStr">
         <is>
-          <t>Beans &amp; Veggie</t>
+          <t>Steak</t>
         </is>
       </c>
       <c r="D126" s="10" t="inlineStr"/>
       <c r="E126" s="10" t="n">
-        <v>9.99</v>
+        <v>12.49</v>
       </c>
       <c r="F126" s="10" t="n"/>
       <c r="G126" s="10" t="n"/>
       <c r="H126" s="10" t="n"/>
       <c r="I126" s="10" t="inlineStr"/>
-      <c r="J126" s="10" t="inlineStr">
-        <is>
-          <t>tacos</t>
-        </is>
-      </c>
+      <c r="J126" s="10" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="9" t="inlineStr">
         <is>
-          <t>tacos/Spicy Chicken</t>
+          <t>tacos/Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="B127" s="10" t="inlineStr">
@@ -5428,23 +5409,27 @@
       </c>
       <c r="C127" s="10" t="inlineStr">
         <is>
-          <t>Spicy Chicken</t>
+          <t>Beans &amp; Veggie</t>
         </is>
       </c>
       <c r="D127" s="10" t="inlineStr"/>
       <c r="E127" s="10" t="n">
-        <v>10.99</v>
+        <v>9.99</v>
       </c>
       <c r="F127" s="10" t="n"/>
       <c r="G127" s="10" t="n"/>
       <c r="H127" s="10" t="n"/>
       <c r="I127" s="10" t="inlineStr"/>
-      <c r="J127" s="10" t="inlineStr"/>
+      <c r="J127" s="10" t="inlineStr">
+        <is>
+          <t>tacos</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="9" t="inlineStr">
         <is>
-          <t>tacos/Ground Beef</t>
+          <t>tacos/Spicy Chicken</t>
         </is>
       </c>
       <c r="B128" s="10" t="inlineStr">
@@ -5454,7 +5439,7 @@
       </c>
       <c r="C128" s="10" t="inlineStr">
         <is>
-          <t>Ground Beef</t>
+          <t>Spicy Chicken</t>
         </is>
       </c>
       <c r="D128" s="10" t="inlineStr"/>
@@ -5470,7 +5455,7 @@
     <row r="129">
       <c r="A129" s="9" t="inlineStr">
         <is>
-          <t>tacos/Zesty Grilled Chicken</t>
+          <t>tacos/Ground Beef</t>
         </is>
       </c>
       <c r="B129" s="10" t="inlineStr">
@@ -5480,7 +5465,7 @@
       </c>
       <c r="C129" s="10" t="inlineStr">
         <is>
-          <t>Zesty Grilled Chicken</t>
+          <t>Ground Beef</t>
         </is>
       </c>
       <c r="D129" s="10" t="inlineStr"/>
@@ -5496,7 +5481,7 @@
     <row r="130">
       <c r="A130" s="9" t="inlineStr">
         <is>
-          <t>tacos/Fish</t>
+          <t>tacos/Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="B130" s="10" t="inlineStr">
@@ -5506,7 +5491,7 @@
       </c>
       <c r="C130" s="10" t="inlineStr">
         <is>
-          <t>Fish</t>
+          <t>Zesty Grilled Chicken</t>
         </is>
       </c>
       <c r="D130" s="10" t="inlineStr"/>
@@ -5522,7 +5507,7 @@
     <row r="131">
       <c r="A131" s="9" t="inlineStr">
         <is>
-          <t>tacos/Shawarma Chicken</t>
+          <t>tacos/Fish</t>
         </is>
       </c>
       <c r="B131" s="10" t="inlineStr">
@@ -5532,12 +5517,12 @@
       </c>
       <c r="C131" s="10" t="inlineStr">
         <is>
-          <t>Shawarma Chicken</t>
+          <t>Fish</t>
         </is>
       </c>
       <c r="D131" s="10" t="inlineStr"/>
       <c r="E131" s="10" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="F131" s="10" t="n"/>
       <c r="G131" s="10" t="n"/>
@@ -5548,7 +5533,7 @@
     <row r="132">
       <c r="A132" s="9" t="inlineStr">
         <is>
-          <t>tacos/Tequila-Lime Glazed Chicken</t>
+          <t>tacos/Shawarma Chicken</t>
         </is>
       </c>
       <c r="B132" s="10" t="inlineStr">
@@ -5558,7 +5543,7 @@
       </c>
       <c r="C132" s="10" t="inlineStr">
         <is>
-          <t>Tequila-Lime Glazed Chicken</t>
+          <t>Shawarma Chicken</t>
         </is>
       </c>
       <c r="D132" s="10" t="inlineStr"/>
@@ -5574,7 +5559,7 @@
     <row r="133">
       <c r="A133" s="9" t="inlineStr">
         <is>
-          <t>tacos/Steak</t>
+          <t>tacos/Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="B133" s="10" t="inlineStr">
@@ -5584,7 +5569,7 @@
       </c>
       <c r="C133" s="10" t="inlineStr">
         <is>
-          <t>Steak</t>
+          <t>Tequila-Lime Glazed Chicken</t>
         </is>
       </c>
       <c r="D133" s="10" t="inlineStr"/>
@@ -5600,22 +5585,22 @@
     <row r="134">
       <c r="A134" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Chips &amp; Salsa — Small</t>
+          <t>tacos/Steak</t>
         </is>
       </c>
       <c r="B134" s="10" t="inlineStr">
         <is>
-          <t>Sides</t>
+          <t>Tacos</t>
         </is>
       </c>
       <c r="C134" s="10" t="inlineStr">
         <is>
-          <t>Chips &amp; Salsa — Small</t>
+          <t>Steak</t>
         </is>
       </c>
       <c r="D134" s="10" t="inlineStr"/>
       <c r="E134" s="10" t="n">
-        <v>2.49</v>
+        <v>11.99</v>
       </c>
       <c r="F134" s="10" t="n"/>
       <c r="G134" s="10" t="n"/>
@@ -5626,7 +5611,7 @@
     <row r="135">
       <c r="A135" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Chips &amp; Salsa — Large</t>
+          <t>burrito-sides/Chips &amp; Salsa — Small</t>
         </is>
       </c>
       <c r="B135" s="10" t="inlineStr">
@@ -5636,12 +5621,12 @@
       </c>
       <c r="C135" s="10" t="inlineStr">
         <is>
-          <t>Chips &amp; Salsa — Large</t>
+          <t>Chips &amp; Salsa — Small</t>
         </is>
       </c>
       <c r="D135" s="10" t="inlineStr"/>
       <c r="E135" s="10" t="n">
-        <v>4.49</v>
+        <v>2.49</v>
       </c>
       <c r="F135" s="10" t="n"/>
       <c r="G135" s="10" t="n"/>
@@ -5652,7 +5637,7 @@
     <row r="136">
       <c r="A136" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Chips &amp; Queso — Small</t>
+          <t>burrito-sides/Chips &amp; Salsa — Large</t>
         </is>
       </c>
       <c r="B136" s="10" t="inlineStr">
@@ -5662,12 +5647,12 @@
       </c>
       <c r="C136" s="10" t="inlineStr">
         <is>
-          <t>Chips &amp; Queso — Small</t>
+          <t>Chips &amp; Salsa — Large</t>
         </is>
       </c>
       <c r="D136" s="10" t="inlineStr"/>
       <c r="E136" s="10" t="n">
-        <v>3.49</v>
+        <v>4.49</v>
       </c>
       <c r="F136" s="10" t="n"/>
       <c r="G136" s="10" t="n"/>
@@ -5678,7 +5663,7 @@
     <row r="137">
       <c r="A137" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Chips &amp; Queso — Large</t>
+          <t>burrito-sides/Chips &amp; Queso — Small</t>
         </is>
       </c>
       <c r="B137" s="10" t="inlineStr">
@@ -5688,12 +5673,12 @@
       </c>
       <c r="C137" s="10" t="inlineStr">
         <is>
-          <t>Chips &amp; Queso — Large</t>
+          <t>Chips &amp; Queso — Small</t>
         </is>
       </c>
       <c r="D137" s="10" t="inlineStr"/>
       <c r="E137" s="10" t="n">
-        <v>6.49</v>
+        <v>3.49</v>
       </c>
       <c r="F137" s="10" t="n"/>
       <c r="G137" s="10" t="n"/>
@@ -5704,7 +5689,7 @@
     <row r="138">
       <c r="A138" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Chips &amp; Guac — Small</t>
+          <t>burrito-sides/Chips &amp; Queso — Large</t>
         </is>
       </c>
       <c r="B138" s="10" t="inlineStr">
@@ -5714,12 +5699,12 @@
       </c>
       <c r="C138" s="10" t="inlineStr">
         <is>
-          <t>Chips &amp; Guac — Small</t>
+          <t>Chips &amp; Queso — Large</t>
         </is>
       </c>
       <c r="D138" s="10" t="inlineStr"/>
       <c r="E138" s="10" t="n">
-        <v>3.99</v>
+        <v>6.49</v>
       </c>
       <c r="F138" s="10" t="n"/>
       <c r="G138" s="10" t="n"/>
@@ -5730,7 +5715,7 @@
     <row r="139">
       <c r="A139" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Chips &amp; Guac — Large</t>
+          <t>burrito-sides/Chips &amp; Guac — Small</t>
         </is>
       </c>
       <c r="B139" s="10" t="inlineStr">
@@ -5740,12 +5725,12 @@
       </c>
       <c r="C139" s="10" t="inlineStr">
         <is>
-          <t>Chips &amp; Guac — Large</t>
+          <t>Chips &amp; Guac — Small</t>
         </is>
       </c>
       <c r="D139" s="10" t="inlineStr"/>
       <c r="E139" s="10" t="n">
-        <v>6.99</v>
+        <v>3.99</v>
       </c>
       <c r="F139" s="10" t="n"/>
       <c r="G139" s="10" t="n"/>
@@ -5756,7 +5741,7 @@
     <row r="140">
       <c r="A140" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Fries Supreme</t>
+          <t>burrito-sides/Chips &amp; Guac — Large</t>
         </is>
       </c>
       <c r="B140" s="10" t="inlineStr">
@@ -5766,12 +5751,12 @@
       </c>
       <c r="C140" s="10" t="inlineStr">
         <is>
-          <t>Fries Supreme</t>
+          <t>Chips &amp; Guac — Large</t>
         </is>
       </c>
       <c r="D140" s="10" t="inlineStr"/>
       <c r="E140" s="10" t="n">
-        <v>9.99</v>
+        <v>6.99</v>
       </c>
       <c r="F140" s="10" t="n"/>
       <c r="G140" s="10" t="n"/>
@@ -5782,7 +5767,7 @@
     <row r="141">
       <c r="A141" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Spicy Fries</t>
+          <t>burrito-sides/Fries Supreme</t>
         </is>
       </c>
       <c r="B141" s="10" t="inlineStr">
@@ -5792,12 +5777,12 @@
       </c>
       <c r="C141" s="10" t="inlineStr">
         <is>
-          <t>Spicy Fries</t>
+          <t>Fries Supreme</t>
         </is>
       </c>
       <c r="D141" s="10" t="inlineStr"/>
       <c r="E141" s="10" t="n">
-        <v>8.99</v>
+        <v>9.99</v>
       </c>
       <c r="F141" s="10" t="n"/>
       <c r="G141" s="10" t="n"/>
@@ -5808,7 +5793,7 @@
     <row r="142">
       <c r="A142" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Deep Fried Pepperoni</t>
+          <t>burrito-sides/Spicy Fries</t>
         </is>
       </c>
       <c r="B142" s="10" t="inlineStr">
@@ -5818,16 +5803,12 @@
       </c>
       <c r="C142" s="10" t="inlineStr">
         <is>
-          <t>Deep Fried Pepperoni</t>
-        </is>
-      </c>
-      <c r="D142" s="10" t="inlineStr">
-        <is>
-          <t>With honey mustard sauce.</t>
-        </is>
-      </c>
+          <t>Spicy Fries</t>
+        </is>
+      </c>
+      <c r="D142" s="10" t="inlineStr"/>
       <c r="E142" s="10" t="n">
-        <v>12.99</v>
+        <v>8.99</v>
       </c>
       <c r="F142" s="10" t="n"/>
       <c r="G142" s="10" t="n"/>
@@ -5838,7 +5819,7 @@
     <row r="143">
       <c r="A143" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Add Chips &amp; Salsa + a Can of Pop</t>
+          <t>burrito-sides/Deep Fried Pepperoni</t>
         </is>
       </c>
       <c r="B143" s="10" t="inlineStr">
@@ -5848,12 +5829,16 @@
       </c>
       <c r="C143" s="10" t="inlineStr">
         <is>
-          <t>Add Chips &amp; Salsa + a Can of Pop</t>
-        </is>
-      </c>
-      <c r="D143" s="10" t="inlineStr"/>
+          <t>Deep Fried Pepperoni</t>
+        </is>
+      </c>
+      <c r="D143" s="10" t="inlineStr">
+        <is>
+          <t>With honey mustard sauce.</t>
+        </is>
+      </c>
       <c r="E143" s="10" t="n">
-        <v>3.49</v>
+        <v>12.99</v>
       </c>
       <c r="F143" s="10" t="n"/>
       <c r="G143" s="10" t="n"/>
@@ -5864,7 +5849,7 @@
     <row r="144">
       <c r="A144" s="9" t="inlineStr">
         <is>
-          <t>burrito-sides/Brownie</t>
+          <t>burrito-sides/Add Chips &amp; Salsa + a Can of Pop</t>
         </is>
       </c>
       <c r="B144" s="10" t="inlineStr">
@@ -5874,12 +5859,12 @@
       </c>
       <c r="C144" s="10" t="inlineStr">
         <is>
-          <t>Brownie</t>
+          <t>Add Chips &amp; Salsa + a Can of Pop</t>
         </is>
       </c>
       <c r="D144" s="10" t="inlineStr"/>
       <c r="E144" s="10" t="n">
-        <v>2.99</v>
+        <v>3.49</v>
       </c>
       <c r="F144" s="10" t="n"/>
       <c r="G144" s="10" t="n"/>
@@ -5887,12 +5872,38 @@
       <c r="I144" s="10" t="inlineStr"/>
       <c r="J144" s="10" t="inlineStr"/>
     </row>
+    <row r="145">
+      <c r="A145" s="9" t="inlineStr">
+        <is>
+          <t>burrito-sides/Brownie</t>
+        </is>
+      </c>
+      <c r="B145" s="10" t="inlineStr">
+        <is>
+          <t>Sides</t>
+        </is>
+      </c>
+      <c r="C145" s="10" t="inlineStr">
+        <is>
+          <t>Brownie</t>
+        </is>
+      </c>
+      <c r="D145" s="10" t="inlineStr"/>
+      <c r="E145" s="10" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="F145" s="10" t="n"/>
+      <c r="G145" s="10" t="n"/>
+      <c r="H145" s="10" t="n"/>
+      <c r="I145" s="10" t="inlineStr"/>
+      <c r="J145" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J5:J144" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the list" error="Pick one from the dropdown, or leave it empty." type="list">
+    <dataValidation sqref="J5:J145" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the list" error="Pick one from the dropdown, or leave it empty." type="list">
       <formula1>=Lists!$B$1:$B$41</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
591ml pop; map pin on the shop itself, in brand red
- Drinks: Any 591ml Pop (was 519ml)
- Shop coordinates from its Google Maps listing (44.698049, -63.4919443);
  the old ones sat ~700 m away at the Main St / Westphal crossroads
- Own red pin with a white ring and soft pulse over the OpenStreetMap
  embed (centred on the shop) instead of OSM's faint green marker

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TastyPizza-Control.xlsx
+++ b/TastyPizza-Control.xlsx
@@ -3809,7 +3809,7 @@
     <row r="76">
       <c r="A76" s="9" t="inlineStr">
         <is>
-          <t>beverages/Any 519ml Pop</t>
+          <t>beverages/Any 591ml Pop</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
@@ -3819,7 +3819,7 @@
       </c>
       <c r="C76" s="10" t="inlineStr">
         <is>
-          <t>Any 519ml Pop</t>
+          <t>Any 591ml Pop</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr"/>

</xml_diff>